<commit_message>
updated codes for combining different pairs
</commit_message>
<xml_diff>
--- a/atomtypes_charges/All_AtomandTopoTypes.xlsx
+++ b/atomtypes_charges/All_AtomandTopoTypes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ornl-my.sharepoint.com/personal/vm5_ornl_gov/Documents/Projects/SingleIonConductors_WithSurface/SIC_Atomistic/atomtypes_charges/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1705" documentId="11_F25DC773A252ABDACC1048D7219A55725ADE5902" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{91725EA8-3855-44ED-B1DA-50CB94E24057}"/>
+  <xr:revisionPtr revIDLastSave="1793" documentId="11_F25DC773A252ABDACC1048D7219A55725ADE5902" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FA05FAF4-14CD-4DA5-8A25-F3E5D6C83E1F}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="All_Unique_Types" sheetId="4" r:id="rId1"/>
@@ -67,7 +67,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1154" uniqueCount="276">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1133" uniqueCount="277">
   <si>
     <t>Do Steps 7 - 10 for angles and dihedrals</t>
   </si>
@@ -893,13 +893,7 @@
     <t>Compile all the UNIQUE PAIR DATA from all the Excel Sheets</t>
   </si>
   <si>
-    <t># Pair Coeffs</t>
-  </si>
-  <si>
     <t>epsilon (kj/mol)</t>
-  </si>
-  <si>
-    <t>sigma (angstrom)</t>
   </si>
   <si>
     <t>NewType_ID-1</t>
@@ -908,16 +902,45 @@
     <t>NewType_ID-2</t>
   </si>
   <si>
-    <t>*</t>
-  </si>
-  <si>
     <t>#Comments</t>
   </si>
   <si>
     <t>Li-LP/Bulk (Table1: https://pubs.acs.org/doi/10.1021/acs.jpcb.3c05591, Wu-Wick)</t>
   </si>
   <si>
-    <t>cut-off</t>
+    <t>Added SHAKE</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>NOTE:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> In most cases, types 23 and 5 are identical and hence type 23 is omitted. Check each time</t>
+    </r>
+  </si>
+  <si>
+    <t>cut-off rc (Angstrom)</t>
+  </si>
+  <si>
+    <t># Pair_Coeffs</t>
+  </si>
+  <si>
+    <t>sigma (Angstrom)</t>
   </si>
 </sst>
 </file>
@@ -952,7 +975,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -977,6 +1000,48 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -991,7 +1056,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1011,6 +1076,18 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1303,7 +1380,8 @@
     <col min="8" max="8" width="11.85546875" customWidth="1"/>
     <col min="9" max="9" width="73.85546875" customWidth="1"/>
     <col min="10" max="10" width="9.140625" customWidth="1"/>
-    <col min="11" max="16" width="18.85546875" customWidth="1"/>
+    <col min="11" max="15" width="18.85546875" customWidth="1"/>
+    <col min="16" max="16" width="21.42578125" customWidth="1"/>
     <col min="17" max="17" width="47.85546875" customWidth="1"/>
     <col min="18" max="20" width="18.85546875" customWidth="1"/>
     <col min="21" max="21" width="10.42578125" customWidth="1"/>
@@ -1452,25 +1530,25 @@
         <v>67</v>
       </c>
       <c r="K2" t="s">
+        <v>275</v>
+      </c>
+      <c r="L2" t="s">
+        <v>268</v>
+      </c>
+      <c r="M2" t="s">
+        <v>269</v>
+      </c>
+      <c r="N2" t="s">
         <v>267</v>
       </c>
-      <c r="L2" t="s">
+      <c r="O2" t="s">
+        <v>276</v>
+      </c>
+      <c r="P2" t="s">
+        <v>274</v>
+      </c>
+      <c r="Q2" t="s">
         <v>270</v>
-      </c>
-      <c r="M2" t="s">
-        <v>271</v>
-      </c>
-      <c r="N2" t="s">
-        <v>268</v>
-      </c>
-      <c r="O2" t="s">
-        <v>269</v>
-      </c>
-      <c r="P2" t="s">
-        <v>275</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>273</v>
       </c>
       <c r="U2" t="s">
         <v>68</v>
@@ -1615,20 +1693,20 @@
       <c r="D3">
         <v>6.9409999999999998</v>
       </c>
-      <c r="E3">
-        <f>B3</f>
-        <v>1</v>
-      </c>
-      <c r="F3">
+      <c r="E3" s="11">
+        <f t="shared" ref="E3:E24" si="0">B3</f>
+        <v>1</v>
+      </c>
+      <c r="F3" s="11">
         <v>2.1510500000000001</v>
       </c>
-      <c r="G3">
+      <c r="G3" s="11">
         <v>2.8</v>
       </c>
-      <c r="H3" t="s">
+      <c r="H3" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="I3" t="s">
+      <c r="I3" s="11" t="s">
         <v>95</v>
       </c>
       <c r="K3" t="s">
@@ -1638,8 +1716,9 @@
         <f>E3</f>
         <v>1</v>
       </c>
-      <c r="M3" s="9" t="s">
-        <v>272</v>
+      <c r="M3" s="9">
+        <f>E3</f>
+        <v>1</v>
       </c>
       <c r="N3">
         <f>F3</f>
@@ -1813,7 +1892,7 @@
     </row>
     <row r="4" spans="1:76" x14ac:dyDescent="0.25">
       <c r="B4">
-        <f t="shared" ref="B4:B11" si="0">B3+1</f>
+        <f t="shared" ref="B4:B11" si="1">B3+1</f>
         <v>2</v>
       </c>
       <c r="C4" t="str">
@@ -1824,48 +1903,49 @@
         <f>PEO_LMP_GMX_UniqueMap!M3</f>
         <v>12.010999999999999</v>
       </c>
-      <c r="E4">
-        <f>B4</f>
+      <c r="E4" s="12">
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="12">
         <f>PEO_LMP_GMX_UniqueMap!J3</f>
         <v>6.6000000000000003E-2</v>
       </c>
-      <c r="G4">
+      <c r="G4" s="12">
         <f>PEO_LMP_GMX_UniqueMap!K3</f>
         <v>3.5</v>
       </c>
-      <c r="H4" t="s">
+      <c r="H4" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="I4" t="s">
+      <c r="I4" s="12" t="s">
         <v>69</v>
       </c>
       <c r="K4" t="s">
         <v>265</v>
       </c>
       <c r="L4">
-        <f t="shared" ref="L4:L25" si="1">E4</f>
+        <f t="shared" ref="L4:L24" si="2">E4</f>
         <v>2</v>
       </c>
-      <c r="M4" s="9" t="s">
-        <v>272</v>
+      <c r="M4" s="9">
+        <f t="shared" ref="M4:M24" si="3">E4</f>
+        <v>2</v>
       </c>
       <c r="N4">
-        <f t="shared" ref="N4:N25" si="2">F4</f>
+        <f t="shared" ref="N4:N24" si="4">F4</f>
         <v>6.6000000000000003E-2</v>
       </c>
       <c r="O4">
-        <f t="shared" ref="O4:O25" si="3">G4</f>
+        <f t="shared" ref="O4:O24" si="5">G4</f>
         <v>3.5</v>
       </c>
       <c r="P4" s="10">
-        <f t="shared" ref="P4:P25" si="4">2.5*O4</f>
+        <f t="shared" ref="P4:P24" si="6">2.5*O4</f>
         <v>8.75</v>
       </c>
       <c r="Q4" t="str">
-        <f t="shared" ref="Q4:Q25" si="5">H4&amp;" "&amp;I4</f>
+        <f t="shared" ref="Q4:Q24" si="7">H4&amp;" "&amp;I4</f>
         <v># C-EO/SEI</v>
       </c>
       <c r="U4">
@@ -1889,29 +1969,30 @@
         <v>C1P</v>
       </c>
       <c r="Z4" t="str">
-        <f t="shared" ref="Z4:Z22" si="6">X4&amp;"-"&amp;Y4</f>
+        <f t="shared" ref="Z4:Z22" si="8">X4&amp;"-"&amp;Y4</f>
         <v>C1P-C1P</v>
       </c>
       <c r="AB4" t="s">
         <v>257</v>
       </c>
-      <c r="AC4">
+      <c r="AC4" s="16">
         <v>2</v>
       </c>
-      <c r="AD4" cm="1">
+      <c r="AD4" s="16" cm="1">
         <f t="array" ref="AD4">_xlfn.XLOOKUP(AG4,$Z$3:$Z$22,ROUND(0.00119502868*$W$3:$W$22,2))</f>
         <v>340</v>
       </c>
-      <c r="AE4" cm="1">
+      <c r="AE4" s="16" cm="1">
         <f t="array" ref="AE4">_xlfn.XLOOKUP(AG4,$Z$3:$Z$22,ROUND(10*$V$3:$V$22,4))</f>
         <v>1.0900000000000001</v>
       </c>
-      <c r="AF4" t="s">
+      <c r="AF4" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="AG4" t="s">
+      <c r="AG4" s="16" t="s">
         <v>121</v>
       </c>
+      <c r="AH4" s="16"/>
       <c r="AM4">
         <f>AM3+1</f>
         <v>2</v>
@@ -1937,7 +2018,7 @@
         <v>C1P</v>
       </c>
       <c r="AS4" t="str">
-        <f t="shared" ref="AS4:AS37" si="7">AP4&amp;"-"&amp;AQ4&amp;"-"&amp;AR4</f>
+        <f t="shared" ref="AS4:AS37" si="9">AP4&amp;"-"&amp;AQ4&amp;"-"&amp;AR4</f>
         <v>O1P-C1P-C1P</v>
       </c>
       <c r="AU4" t="s">
@@ -1989,7 +2070,7 @@
         <v>0</v>
       </c>
       <c r="BL4">
-        <f t="shared" ref="BL4:BL33" si="8">SUM(BF4:BK4)</f>
+        <f t="shared" ref="BL4:BL33" si="10">SUM(BF4:BK4)</f>
         <v>0</v>
       </c>
       <c r="BM4" t="str">
@@ -2027,7 +2108,7 @@
     </row>
     <row r="5" spans="1:76" x14ac:dyDescent="0.25">
       <c r="B5">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>3</v>
       </c>
       <c r="C5" t="str">
@@ -2038,52 +2119,53 @@
         <f>PEO_LMP_GMX_UniqueMap!M5</f>
         <v>1.008</v>
       </c>
-      <c r="E5">
-        <f>B5</f>
-        <v>3</v>
-      </c>
-      <c r="F5">
+      <c r="E5" s="12">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="F5" s="12">
         <f>PEO_LMP_GMX_UniqueMap!J5</f>
         <v>0.03</v>
       </c>
-      <c r="G5">
+      <c r="G5" s="12">
         <f>PEO_LMP_GMX_UniqueMap!K5</f>
         <v>2.5</v>
       </c>
-      <c r="H5" t="s">
+      <c r="H5" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="I5" t="s">
+      <c r="I5" s="12" t="s">
         <v>70</v>
       </c>
       <c r="K5" t="s">
         <v>265</v>
       </c>
       <c r="L5">
-        <f t="shared" si="1"/>
-        <v>3</v>
-      </c>
-      <c r="M5" s="9" t="s">
-        <v>272</v>
+        <f t="shared" si="2"/>
+        <v>3</v>
+      </c>
+      <c r="M5" s="9">
+        <f t="shared" si="3"/>
+        <v>3</v>
       </c>
       <c r="N5">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.03</v>
       </c>
       <c r="O5">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>2.5</v>
       </c>
       <c r="P5" s="10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>6.25</v>
       </c>
       <c r="Q5" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v># H-EO/SEI</v>
       </c>
       <c r="U5">
-        <f t="shared" ref="U5:U22" si="9">U4+1</f>
+        <f t="shared" ref="U5:U22" si="11">U4+1</f>
         <v>3</v>
       </c>
       <c r="V5">
@@ -2103,7 +2185,7 @@
         <v>C1P</v>
       </c>
       <c r="Z5" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>HP-C1P</v>
       </c>
       <c r="AB5" t="s">
@@ -2127,7 +2209,7 @@
         <v>122</v>
       </c>
       <c r="AM5">
-        <f t="shared" ref="AM5:AM37" si="10">AM4+1</f>
+        <f t="shared" ref="AM5:AM37" si="12">AM4+1</f>
         <v>3</v>
       </c>
       <c r="AN5">
@@ -2151,7 +2233,7 @@
         <v>HP</v>
       </c>
       <c r="AS5" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>O1P-C1P-HP</v>
       </c>
       <c r="AU5" t="s">
@@ -2175,7 +2257,7 @@
         <v>138</v>
       </c>
       <c r="BE5">
-        <f t="shared" ref="BE5:BE43" si="11">BE4+1</f>
+        <f t="shared" ref="BE5:BE43" si="13">BE4+1</f>
         <v>3</v>
       </c>
       <c r="BF5">
@@ -2203,7 +2285,7 @@
         <v>0</v>
       </c>
       <c r="BL5">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="BM5" t="str">
@@ -2241,7 +2323,7 @@
     </row>
     <row r="6" spans="1:76" x14ac:dyDescent="0.25">
       <c r="B6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="C6" t="str">
@@ -2252,52 +2334,53 @@
         <f>PEO_LMP_GMX_UniqueMap!M4</f>
         <v>15.999000000000001</v>
       </c>
-      <c r="E6">
-        <f>B6</f>
+      <c r="E6" s="12">
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="F6">
+      <c r="F6" s="12">
         <f>PEO_LMP_GMX_UniqueMap!J4</f>
         <v>0.14000000000000001</v>
       </c>
-      <c r="G6">
+      <c r="G6" s="12">
         <f>PEO_LMP_GMX_UniqueMap!K4</f>
         <v>2.9</v>
       </c>
-      <c r="H6" t="s">
+      <c r="H6" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="I6" t="s">
+      <c r="I6" s="12" t="s">
         <v>71</v>
       </c>
       <c r="K6" t="s">
         <v>265</v>
       </c>
       <c r="L6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>4</v>
       </c>
-      <c r="M6" s="9" t="s">
-        <v>272</v>
+      <c r="M6" s="9">
+        <f t="shared" si="3"/>
+        <v>4</v>
       </c>
       <c r="N6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.14000000000000001</v>
       </c>
       <c r="O6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>2.9</v>
       </c>
       <c r="P6" s="10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>7.25</v>
       </c>
       <c r="Q6" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v># O-EO/SEI</v>
       </c>
       <c r="U6">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>4</v>
       </c>
       <c r="V6">
@@ -2317,7 +2400,7 @@
         <v>O1C</v>
       </c>
       <c r="Z6" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>C1C-O1C</v>
       </c>
       <c r="AB6" t="s">
@@ -2341,7 +2424,7 @@
         <v>108</v>
       </c>
       <c r="AM6">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>4</v>
       </c>
       <c r="AN6">
@@ -2365,31 +2448,31 @@
         <v>HP</v>
       </c>
       <c r="AS6" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>C1P-C1P-HP</v>
       </c>
       <c r="AU6" t="s">
         <v>260</v>
       </c>
-      <c r="AV6">
+      <c r="AV6" s="16">
         <v>4</v>
       </c>
-      <c r="AW6" cm="1">
+      <c r="AW6" s="16" cm="1">
         <f t="array" ref="AW6">_xlfn.XLOOKUP(AZ6,$AS$3:$AS$37,ROUND(0.119502868*$AO$3:$AO$37,3))</f>
         <v>33</v>
       </c>
-      <c r="AX6" cm="1">
+      <c r="AX6" s="16" cm="1">
         <f t="array" ref="AX6">_xlfn.XLOOKUP(AZ6,$AS$3:$AS$37,ROUND($AN$3:$AN$37,3))</f>
         <v>107.8</v>
       </c>
-      <c r="AY6" t="s">
+      <c r="AY6" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="AZ6" t="s">
+      <c r="AZ6" s="16" t="s">
         <v>139</v>
       </c>
       <c r="BE6">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>4</v>
       </c>
       <c r="BF6">
@@ -2417,7 +2500,7 @@
         <v>0</v>
       </c>
       <c r="BL6">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>-8.8817841970012523E-16</v>
       </c>
       <c r="BM6" t="str">
@@ -2455,59 +2538,60 @@
     </row>
     <row r="7" spans="1:76" x14ac:dyDescent="0.25">
       <c r="B7">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="C7" t="s">
+        <v>90</v>
+      </c>
+      <c r="D7">
+        <v>6.9409999999999998</v>
+      </c>
+      <c r="E7" s="13">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="C7" t="s">
-        <v>90</v>
-      </c>
-      <c r="D7">
-        <v>6.9409999999999998</v>
-      </c>
-      <c r="E7">
-        <f>B7</f>
-        <v>5</v>
-      </c>
-      <c r="F7">
+      <c r="F7" s="13">
         <v>0.4</v>
       </c>
-      <c r="G7">
+      <c r="G7" s="13">
         <v>1.4</v>
       </c>
-      <c r="H7" t="s">
+      <c r="H7" s="13" t="s">
         <v>68</v>
       </c>
-      <c r="I7" t="s">
+      <c r="I7" s="13" t="s">
         <v>89</v>
       </c>
       <c r="K7" t="s">
         <v>265</v>
       </c>
       <c r="L7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>5</v>
       </c>
-      <c r="M7" s="9" t="s">
-        <v>272</v>
+      <c r="M7" s="9">
+        <f t="shared" si="3"/>
+        <v>5</v>
       </c>
       <c r="N7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.4</v>
       </c>
       <c r="O7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>1.4</v>
       </c>
       <c r="P7" s="10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>3.5</v>
       </c>
       <c r="Q7" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v># Li-LP/SEI (Table1: https://pubs.acs.org/doi/10.1021/acs.jpcb.3c05591, Wu-Wick)</v>
       </c>
       <c r="U7">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>5</v>
       </c>
       <c r="V7">
@@ -2527,7 +2611,7 @@
         <v>C1C</v>
       </c>
       <c r="Z7" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>O2C-C1C</v>
       </c>
       <c r="AB7" t="s">
@@ -2551,7 +2635,7 @@
         <v>123</v>
       </c>
       <c r="AM7">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>5</v>
       </c>
       <c r="AN7">
@@ -2575,7 +2659,7 @@
         <v>HP</v>
       </c>
       <c r="AS7" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>HP-C1P-HP</v>
       </c>
       <c r="AU7" t="s">
@@ -2599,7 +2683,7 @@
         <v>167</v>
       </c>
       <c r="BE7">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>5</v>
       </c>
       <c r="BF7">
@@ -2627,7 +2711,7 @@
         <v>0</v>
       </c>
       <c r="BL7">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="BM7" t="str">
@@ -2665,7 +2749,7 @@
     </row>
     <row r="8" spans="1:76" x14ac:dyDescent="0.25">
       <c r="B8">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>6</v>
       </c>
       <c r="C8" t="str">
@@ -2676,55 +2760,56 @@
         <f>CO32M_LMP_GMX_UniqueMap!M4</f>
         <v>12.010999999999999</v>
       </c>
-      <c r="E8">
-        <f>B8</f>
+      <c r="E8" s="14">
+        <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="F8">
+      <c r="F8" s="14">
         <f>CO32M_LMP_GMX_UniqueMap!J4</f>
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="G8">
+      <c r="G8" s="14">
         <f>CO32M_LMP_GMX_UniqueMap!K4</f>
         <v>3.55</v>
       </c>
-      <c r="H8" t="s">
+      <c r="H8" s="14" t="s">
         <v>68</v>
       </c>
-      <c r="I8" t="s">
+      <c r="I8" s="14" t="s">
         <v>72</v>
       </c>
       <c r="K8" t="s">
         <v>265</v>
       </c>
       <c r="L8">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>6</v>
       </c>
-      <c r="M8" s="9" t="s">
-        <v>272</v>
+      <c r="M8" s="9">
+        <f t="shared" si="3"/>
+        <v>6</v>
       </c>
       <c r="N8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="O8">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>3.55</v>
       </c>
       <c r="P8" s="10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>8.875</v>
       </c>
       <c r="Q8" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v># C1-COI/SEI</v>
       </c>
       <c r="R8" s="6"/>
       <c r="S8" s="6"/>
       <c r="T8" s="6"/>
       <c r="U8">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>6</v>
       </c>
       <c r="V8">
@@ -2744,7 +2829,7 @@
         <v>HMT</v>
       </c>
       <c r="Z8" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>C1MT-HMT</v>
       </c>
       <c r="AB8" t="s">
@@ -2768,7 +2853,7 @@
         <v>109</v>
       </c>
       <c r="AM8">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>6</v>
       </c>
       <c r="AN8">
@@ -2792,7 +2877,7 @@
         <v>O2C</v>
       </c>
       <c r="AS8" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>O1C-C1C-O2C</v>
       </c>
       <c r="AU8" t="s">
@@ -2816,7 +2901,7 @@
         <v>140</v>
       </c>
       <c r="BE8">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>6</v>
       </c>
       <c r="BF8">
@@ -2844,7 +2929,7 @@
         <v>0</v>
       </c>
       <c r="BL8">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="BM8" t="str">
@@ -2862,15 +2947,15 @@
         <v>1.3</v>
       </c>
       <c r="BS8" s="7">
-        <f t="shared" ref="BS8:BU8" si="12">BS62</f>
+        <f t="shared" ref="BS8:BU8" si="14">BS62</f>
         <v>-0.2</v>
       </c>
       <c r="BT8" s="7">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v>0.2</v>
       </c>
       <c r="BU8" s="7">
-        <f t="shared" si="12"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="BV8" s="7" t="s">
@@ -2885,7 +2970,7 @@
     </row>
     <row r="9" spans="1:76" x14ac:dyDescent="0.25">
       <c r="B9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>7</v>
       </c>
       <c r="C9" t="str">
@@ -2896,52 +2981,53 @@
         <f>CO32M_LMP_GMX_UniqueMap!M3</f>
         <v>15.999000000000001</v>
       </c>
-      <c r="E9">
-        <f>B9</f>
+      <c r="E9" s="14">
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="F9">
+      <c r="F9" s="14">
         <f>CO32M_LMP_GMX_UniqueMap!J3</f>
         <v>0.21</v>
       </c>
-      <c r="G9">
+      <c r="G9" s="14">
         <f>CO32M_LMP_GMX_UniqueMap!K3</f>
         <v>2.96</v>
       </c>
-      <c r="H9" t="s">
+      <c r="H9" s="14" t="s">
         <v>68</v>
       </c>
-      <c r="I9" t="s">
+      <c r="I9" s="14" t="s">
         <v>73</v>
       </c>
       <c r="K9" t="s">
         <v>265</v>
       </c>
       <c r="L9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>7</v>
       </c>
-      <c r="M9" s="9" t="s">
-        <v>272</v>
+      <c r="M9" s="9">
+        <f t="shared" si="3"/>
+        <v>7</v>
       </c>
       <c r="N9">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.21</v>
       </c>
       <c r="O9">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>2.96</v>
       </c>
       <c r="P9" s="10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>7.4</v>
       </c>
       <c r="Q9" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v># O1-COI/SEI</v>
       </c>
       <c r="U9">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>7</v>
       </c>
       <c r="V9">
@@ -2961,7 +3047,7 @@
         <v>C2MT</v>
       </c>
       <c r="Z9" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>O2MT-C2MT</v>
       </c>
       <c r="AB9" t="s">
@@ -2989,7 +3075,7 @@
         <v>Same as C1MT-C1MT</v>
       </c>
       <c r="AM9">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>7</v>
       </c>
       <c r="AN9">
@@ -3013,7 +3099,7 @@
         <v>O2C</v>
       </c>
       <c r="AS9" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>O2C-C1C-O2C</v>
       </c>
       <c r="AU9" t="s">
@@ -3037,7 +3123,7 @@
         <v>141</v>
       </c>
       <c r="BE9">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>7</v>
       </c>
       <c r="BF9">
@@ -3065,7 +3151,7 @@
         <v>0</v>
       </c>
       <c r="BL9">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>-8.8817841970012523E-16</v>
       </c>
       <c r="BM9" t="str">
@@ -3083,15 +3169,15 @@
         <v>1.3</v>
       </c>
       <c r="BS9" s="7">
-        <f t="shared" ref="BS9:BU9" si="13">BS62</f>
+        <f t="shared" ref="BS9:BU9" si="15">BS62</f>
         <v>-0.2</v>
       </c>
       <c r="BT9" s="7">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>0.2</v>
       </c>
       <c r="BU9" s="7">
-        <f t="shared" si="13"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="BV9" s="7" t="s">
@@ -3106,7 +3192,7 @@
     </row>
     <row r="10" spans="1:76" x14ac:dyDescent="0.25">
       <c r="B10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>8</v>
       </c>
       <c r="C10" t="str">
@@ -3117,52 +3203,53 @@
         <f>CO32M_LMP_GMX_UniqueMap!M5</f>
         <v>15.999000000000001</v>
       </c>
-      <c r="E10">
-        <f>B10</f>
+      <c r="E10" s="14">
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="F10">
+      <c r="F10" s="14">
         <f>CO32M_LMP_GMX_UniqueMap!J5</f>
         <v>0.17</v>
       </c>
-      <c r="G10">
+      <c r="G10" s="14">
         <f>CO32M_LMP_GMX_UniqueMap!K5</f>
         <v>3.12</v>
       </c>
-      <c r="H10" t="s">
+      <c r="H10" s="14" t="s">
         <v>68</v>
       </c>
-      <c r="I10" t="s">
+      <c r="I10" s="14" t="s">
         <v>74</v>
       </c>
       <c r="K10" t="s">
         <v>265</v>
       </c>
       <c r="L10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>8</v>
       </c>
-      <c r="M10" s="9" t="s">
-        <v>272</v>
+      <c r="M10" s="9">
+        <f t="shared" si="3"/>
+        <v>8</v>
       </c>
       <c r="N10">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.17</v>
       </c>
       <c r="O10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>3.12</v>
       </c>
       <c r="P10" s="10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>7.8000000000000007</v>
       </c>
       <c r="Q10" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v># O2-COI/SEI</v>
       </c>
       <c r="U10">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>8</v>
       </c>
       <c r="V10">
@@ -3182,7 +3269,7 @@
         <v>C2MT</v>
       </c>
       <c r="Z10" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>O1MT-C2MT</v>
       </c>
       <c r="AB10" t="s">
@@ -3206,7 +3293,7 @@
         <v>125</v>
       </c>
       <c r="AM10">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>8</v>
       </c>
       <c r="AN10">
@@ -3230,7 +3317,7 @@
         <v>NMT</v>
       </c>
       <c r="AS10" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>C1MT-SMT-NMT</v>
       </c>
       <c r="AU10" t="s">
@@ -3254,7 +3341,7 @@
         <v>142</v>
       </c>
       <c r="BE10">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>8</v>
       </c>
       <c r="BF10">
@@ -3282,7 +3369,7 @@
         <v>0</v>
       </c>
       <c r="BL10">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>1.000000000000334E-3</v>
       </c>
       <c r="BM10" t="str">
@@ -3300,15 +3387,15 @@
         <v>-2.06</v>
       </c>
       <c r="BS10" s="7">
-        <f t="shared" ref="BS10:BU10" si="14">BS63</f>
+        <f t="shared" ref="BS10:BU10" si="16">BS63</f>
         <v>-0.313</v>
       </c>
       <c r="BT10" s="7">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>0.315</v>
       </c>
       <c r="BU10" s="7">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>0</v>
       </c>
       <c r="BV10" s="7" t="s">
@@ -3323,7 +3410,7 @@
     </row>
     <row r="11" spans="1:76" x14ac:dyDescent="0.25">
       <c r="B11">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>9</v>
       </c>
       <c r="C11" t="str">
@@ -3334,52 +3421,53 @@
         <f>MTFSI_LMP_GMX_UniqueMap!M5</f>
         <v>12.010999999999999</v>
       </c>
-      <c r="E11">
-        <f>B11</f>
+      <c r="E11" s="15">
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="F11">
+      <c r="F11" s="15">
         <f>MTFSI_LMP_GMX_UniqueMap!J5</f>
         <v>6.6000000000000003E-2</v>
       </c>
-      <c r="G11">
+      <c r="G11" s="15">
         <f>MTFSI_LMP_GMX_UniqueMap!K5</f>
         <v>3.5</v>
       </c>
-      <c r="H11" t="s">
+      <c r="H11" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="I11" t="s">
+      <c r="I11" s="15" t="s">
         <v>75</v>
       </c>
       <c r="K11" t="s">
         <v>265</v>
       </c>
       <c r="L11">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>9</v>
       </c>
-      <c r="M11" s="9" t="s">
-        <v>272</v>
+      <c r="M11" s="9">
+        <f t="shared" si="3"/>
+        <v>9</v>
       </c>
       <c r="N11">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>6.6000000000000003E-2</v>
       </c>
       <c r="O11">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>3.5</v>
       </c>
       <c r="P11" s="10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>8.75</v>
       </c>
       <c r="Q11" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v># C1-MT/Bulk</v>
       </c>
       <c r="U11">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>9</v>
       </c>
       <c r="V11">
@@ -3399,7 +3487,7 @@
         <v>C1MT</v>
       </c>
       <c r="Z11" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>FMT-C1MT</v>
       </c>
       <c r="AB11" t="s">
@@ -3423,7 +3511,7 @@
         <v>126</v>
       </c>
       <c r="AM11">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>9</v>
       </c>
       <c r="AN11">
@@ -3447,7 +3535,7 @@
         <v>O3MT</v>
       </c>
       <c r="AS11" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>NMT-SMT-O3MT</v>
       </c>
       <c r="AU11" t="s">
@@ -3474,7 +3562,7 @@
         <v>176</v>
       </c>
       <c r="BE11">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>9</v>
       </c>
       <c r="BF11">
@@ -3502,7 +3590,7 @@
         <v>0</v>
       </c>
       <c r="BL11">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="BM11" t="str">
@@ -3550,52 +3638,53 @@
         <f>VEC_LMP_GMX_UniqueMap!M6</f>
         <v>12.010999999999999</v>
       </c>
-      <c r="E12">
-        <f>B12</f>
+      <c r="E12" s="15">
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="F12">
+      <c r="F12" s="15">
         <f>VEC_LMP_GMX_UniqueMap!J6</f>
         <v>6.6000000000000003E-2</v>
       </c>
-      <c r="G12">
+      <c r="G12" s="15">
         <f>VEC_LMP_GMX_UniqueMap!K6</f>
         <v>3.5</v>
       </c>
-      <c r="H12" t="s">
+      <c r="H12" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="I12" t="s">
+      <c r="I12" s="15" t="s">
         <v>76</v>
       </c>
       <c r="K12" t="s">
         <v>265</v>
       </c>
       <c r="L12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>10</v>
       </c>
-      <c r="M12" s="9" t="s">
-        <v>272</v>
+      <c r="M12" s="9">
+        <f t="shared" si="3"/>
+        <v>10</v>
       </c>
       <c r="N12">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>6.6000000000000003E-2</v>
       </c>
       <c r="O12">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>3.5</v>
       </c>
       <c r="P12" s="10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>8.75</v>
       </c>
       <c r="Q12" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v># C1-VEC/Bulk</v>
       </c>
       <c r="U12">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>10</v>
       </c>
       <c r="V12">
@@ -3615,31 +3704,31 @@
         <v>O1MT</v>
       </c>
       <c r="Z12" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>C1MT-O1MT</v>
       </c>
       <c r="AB12" t="s">
         <v>257</v>
       </c>
-      <c r="AC12">
+      <c r="AC12" s="16">
         <v>10</v>
       </c>
-      <c r="AD12" cm="1">
+      <c r="AD12" s="16" cm="1">
         <f t="array" ref="AD12">_xlfn.XLOOKUP(AG12,$Z$3:$Z$22,ROUND(0.00119502868*$W$3:$W$22,2))</f>
         <v>340</v>
       </c>
-      <c r="AE12" cm="1">
+      <c r="AE12" s="16" cm="1">
         <f t="array" ref="AE12">_xlfn.XLOOKUP(AG12,$Z$3:$Z$22,ROUND(10*$V$3:$V$22,4))</f>
         <v>1.0900000000000001</v>
       </c>
-      <c r="AF12" t="s">
+      <c r="AF12" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="AG12" t="s">
+      <c r="AG12" s="16" t="s">
         <v>110</v>
       </c>
       <c r="AM12">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>10</v>
       </c>
       <c r="AN12">
@@ -3663,7 +3752,7 @@
         <v>HMT</v>
       </c>
       <c r="AS12" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>HMT-C1MT-HMT</v>
       </c>
       <c r="AU12" t="s">
@@ -3687,7 +3776,7 @@
         <v>144</v>
       </c>
       <c r="BE12">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>10</v>
       </c>
       <c r="BF12">
@@ -3715,7 +3804,7 @@
         <v>0</v>
       </c>
       <c r="BL12">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>-4.4408920985006262E-16</v>
       </c>
       <c r="BM12" t="str">
@@ -3763,52 +3852,53 @@
         <f>MTFSI_LMP_GMX_UniqueMap!M6</f>
         <v>12.010999999999999</v>
       </c>
-      <c r="E13">
-        <f>B13</f>
+      <c r="E13" s="15">
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="F13">
+      <c r="F13" s="15">
         <f>MTFSI_LMP_GMX_UniqueMap!J6</f>
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="G13">
+      <c r="G13" s="15">
         <f>MTFSI_LMP_GMX_UniqueMap!K6</f>
         <v>3.55</v>
       </c>
-      <c r="H13" t="s">
+      <c r="H13" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="I13" t="s">
+      <c r="I13" s="15" t="s">
         <v>77</v>
       </c>
       <c r="K13" t="s">
         <v>265</v>
       </c>
       <c r="L13">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>11</v>
       </c>
-      <c r="M13" s="9" t="s">
-        <v>272</v>
+      <c r="M13" s="9">
+        <f t="shared" si="3"/>
+        <v>11</v>
       </c>
       <c r="N13">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="O13">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>3.55</v>
       </c>
       <c r="P13" s="10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>8.875</v>
       </c>
       <c r="Q13" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v># C2-MT/Bulk</v>
       </c>
       <c r="U13">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>11</v>
       </c>
       <c r="V13">
@@ -3828,7 +3918,7 @@
         <v>SMT</v>
       </c>
       <c r="Z13" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>O3MT-SMT</v>
       </c>
       <c r="AB13" t="s">
@@ -3852,7 +3942,7 @@
         <v>111</v>
       </c>
       <c r="AM13">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>11</v>
       </c>
       <c r="AN13">
@@ -3876,31 +3966,31 @@
         <v>SMT</v>
       </c>
       <c r="AS13" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>C1MT-C1MT-SMT</v>
       </c>
       <c r="AU13" t="s">
         <v>260</v>
       </c>
-      <c r="AV13">
+      <c r="AV13" s="16">
         <v>11</v>
       </c>
-      <c r="AW13" cm="1">
+      <c r="AW13" s="16" cm="1">
         <f t="array" ref="AW13">_xlfn.XLOOKUP(AZ13,$AS$3:$AS$37,ROUND(0.119502868*$AO$3:$AO$37,3))</f>
         <v>37.5</v>
       </c>
-      <c r="AX13" cm="1">
+      <c r="AX13" s="16" cm="1">
         <f t="array" ref="AX13">_xlfn.XLOOKUP(AZ13,$AS$3:$AS$37,ROUND($AN$3:$AN$37,3))</f>
         <v>110.7</v>
       </c>
-      <c r="AY13" t="s">
+      <c r="AY13" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="AZ13" t="s">
+      <c r="AZ13" s="16" t="s">
         <v>168</v>
       </c>
       <c r="BE13">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>11</v>
       </c>
       <c r="BF13">
@@ -3928,7 +4018,7 @@
         <v>0</v>
       </c>
       <c r="BL13">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>-1.0000000000012221E-3</v>
       </c>
       <c r="BM13" t="str">
@@ -3976,52 +4066,53 @@
         <f>VEC_LMP_GMX_UniqueMap!M7</f>
         <v>12.010999999999999</v>
       </c>
-      <c r="E14">
-        <f>B14</f>
+      <c r="E14" s="15">
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="F14">
+      <c r="F14" s="15">
         <f>VEC_LMP_GMX_UniqueMap!J7</f>
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="G14">
+      <c r="G14" s="15">
         <f>VEC_LMP_GMX_UniqueMap!K7</f>
         <v>3.55</v>
       </c>
-      <c r="H14" t="s">
+      <c r="H14" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="I14" t="s">
+      <c r="I14" s="15" t="s">
         <v>78</v>
       </c>
       <c r="K14" t="s">
         <v>265</v>
       </c>
       <c r="L14">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>12</v>
       </c>
-      <c r="M14" s="9" t="s">
-        <v>272</v>
+      <c r="M14" s="9">
+        <f t="shared" si="3"/>
+        <v>12</v>
       </c>
       <c r="N14">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="O14">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>3.55</v>
       </c>
       <c r="P14" s="10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>8.875</v>
       </c>
       <c r="Q14" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v># C2-VEC/Bulk</v>
       </c>
       <c r="U14">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>12</v>
       </c>
       <c r="V14">
@@ -4041,7 +4132,7 @@
         <v>C1MT</v>
       </c>
       <c r="Z14" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>C2MT-C1MT</v>
       </c>
       <c r="AB14" t="s">
@@ -4065,7 +4156,7 @@
         <v>127</v>
       </c>
       <c r="AM14">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>12</v>
       </c>
       <c r="AN14">
@@ -4089,7 +4180,7 @@
         <v>O3MT</v>
       </c>
       <c r="AS14" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>C1MT-SMT-O3MT</v>
       </c>
       <c r="AU14" t="s">
@@ -4113,7 +4204,7 @@
         <v>169</v>
       </c>
       <c r="BE14">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>12</v>
       </c>
       <c r="BF14">
@@ -4141,7 +4232,7 @@
         <v>0</v>
       </c>
       <c r="BL14">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="BM14" t="str">
@@ -4159,15 +4250,15 @@
         <v>1.3</v>
       </c>
       <c r="BS14" s="7">
-        <f t="shared" ref="BS14:BU14" si="15">BS62</f>
+        <f t="shared" ref="BS14:BU14" si="17">BS62</f>
         <v>-0.2</v>
       </c>
       <c r="BT14" s="7">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>0.2</v>
       </c>
       <c r="BU14" s="7">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="BV14" s="7" t="s">
@@ -4192,52 +4283,53 @@
         <f>MTFSI_LMP_GMX_UniqueMap!M4</f>
         <v>18.998000000000001</v>
       </c>
-      <c r="E15">
-        <f>B15</f>
+      <c r="E15" s="15">
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="F15">
+      <c r="F15" s="15">
         <f>MTFSI_LMP_GMX_UniqueMap!J4</f>
         <v>0.06</v>
       </c>
-      <c r="G15">
+      <c r="G15" s="15">
         <f>MTFSI_LMP_GMX_UniqueMap!K4</f>
         <v>2.9</v>
       </c>
-      <c r="H15" t="s">
+      <c r="H15" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="I15" t="s">
+      <c r="I15" s="15" t="s">
         <v>79</v>
       </c>
       <c r="K15" t="s">
         <v>265</v>
       </c>
       <c r="L15">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>13</v>
       </c>
-      <c r="M15" s="9" t="s">
-        <v>272</v>
+      <c r="M15" s="9">
+        <f t="shared" si="3"/>
+        <v>13</v>
       </c>
       <c r="N15">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.06</v>
       </c>
       <c r="O15">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>2.9</v>
       </c>
       <c r="P15" s="10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>7.25</v>
       </c>
       <c r="Q15" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v># F-MT/Bulk</v>
       </c>
       <c r="U15">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>13</v>
       </c>
       <c r="V15">
@@ -4257,7 +4349,7 @@
         <v>C1MT</v>
       </c>
       <c r="Z15" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>C1MT-C1MT</v>
       </c>
       <c r="AB15" t="s">
@@ -4281,7 +4373,7 @@
         <v>112</v>
       </c>
       <c r="AM15">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>13</v>
       </c>
       <c r="AN15">
@@ -4305,7 +4397,7 @@
         <v>FMT</v>
       </c>
       <c r="AS15" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>FMT-C1MT-FMT</v>
       </c>
       <c r="AU15" t="s">
@@ -4329,7 +4421,7 @@
         <v>145</v>
       </c>
       <c r="BE15">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>13</v>
       </c>
       <c r="BF15">
@@ -4357,7 +4449,7 @@
         <v>0</v>
       </c>
       <c r="BL15">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="BM15" t="str">
@@ -4375,15 +4467,15 @@
         <v>0</v>
       </c>
       <c r="BS15" s="7">
-        <f t="shared" ref="BS15:BU15" si="16">BS11</f>
+        <f t="shared" ref="BS15:BU15" si="18">BS11</f>
         <v>0</v>
       </c>
       <c r="BT15" s="7">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>0.3</v>
       </c>
       <c r="BU15" s="7">
-        <f t="shared" si="16"/>
+        <f t="shared" si="18"/>
         <v>0</v>
       </c>
       <c r="BV15" s="7" t="s">
@@ -4409,52 +4501,53 @@
         <f>MTFSI_LMP_GMX_UniqueMap!M3</f>
         <v>1.008</v>
       </c>
-      <c r="E16">
-        <f>B16</f>
+      <c r="E16" s="15">
+        <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="F16">
+      <c r="F16" s="15">
         <f>MTFSI_LMP_GMX_UniqueMap!J3</f>
         <v>0.03</v>
       </c>
-      <c r="G16">
+      <c r="G16" s="15">
         <f>MTFSI_LMP_GMX_UniqueMap!K3</f>
         <v>2.5</v>
       </c>
-      <c r="H16" t="s">
+      <c r="H16" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="I16" t="s">
+      <c r="I16" s="15" t="s">
         <v>80</v>
       </c>
       <c r="K16" t="s">
         <v>265</v>
       </c>
       <c r="L16">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>14</v>
       </c>
-      <c r="M16" s="9" t="s">
-        <v>272</v>
+      <c r="M16" s="9">
+        <f t="shared" si="3"/>
+        <v>14</v>
       </c>
       <c r="N16">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.03</v>
       </c>
       <c r="O16">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>2.5</v>
       </c>
       <c r="P16" s="10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>6.25</v>
       </c>
       <c r="Q16" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v># H-M/Bulk</v>
       </c>
       <c r="U16">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>14</v>
       </c>
       <c r="V16">
@@ -4474,31 +4567,31 @@
         <v>SMT</v>
       </c>
       <c r="Z16" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>NMT-SMT</v>
       </c>
       <c r="AB16" t="s">
         <v>257</v>
       </c>
-      <c r="AC16">
+      <c r="AC16" s="16">
         <v>14</v>
       </c>
-      <c r="AD16" cm="1">
+      <c r="AD16" s="16" cm="1">
         <f t="array" ref="AD16">_xlfn.XLOOKUP(AG16,$Z$3:$Z$22,ROUND(0.00119502868*$W$3:$W$22,2))</f>
         <v>340</v>
       </c>
-      <c r="AE16" cm="1">
+      <c r="AE16" s="16" cm="1">
         <f t="array" ref="AE16">_xlfn.XLOOKUP(AG16,$Z$3:$Z$22,ROUND(10*$V$3:$V$22,4))</f>
         <v>1.0900000000000001</v>
       </c>
-      <c r="AF16" t="s">
+      <c r="AF16" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="AG16" t="s">
+      <c r="AG16" s="16" t="s">
         <v>113</v>
       </c>
       <c r="AM16">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>14</v>
       </c>
       <c r="AN16">
@@ -4522,7 +4615,7 @@
         <v>C1MT</v>
       </c>
       <c r="AS16" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>O1MT-C1MT-C1MT</v>
       </c>
       <c r="AU16" t="s">
@@ -4549,7 +4642,7 @@
         <v>176</v>
       </c>
       <c r="BE16">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>14</v>
       </c>
       <c r="BF16">
@@ -4577,7 +4670,7 @@
         <v>0</v>
       </c>
       <c r="BL16">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="BM16" t="str">
@@ -4626,52 +4719,53 @@
         <f>VEC_LMP_GMX_UniqueMap!M3</f>
         <v>1.008</v>
       </c>
-      <c r="E17">
-        <f>B17</f>
+      <c r="E17" s="15">
+        <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="F17">
+      <c r="F17" s="15">
         <f>VEC_LMP_GMX_UniqueMap!J3</f>
         <v>0.03</v>
       </c>
-      <c r="G17">
+      <c r="G17" s="15">
         <f>VEC_LMP_GMX_UniqueMap!K3</f>
         <v>2.5</v>
       </c>
-      <c r="H17" t="s">
+      <c r="H17" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="I17" t="s">
+      <c r="I17" s="15" t="s">
         <v>81</v>
       </c>
       <c r="K17" t="s">
         <v>265</v>
       </c>
       <c r="L17">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>15</v>
       </c>
-      <c r="M17" s="9" t="s">
-        <v>272</v>
+      <c r="M17" s="9">
+        <f t="shared" si="3"/>
+        <v>15</v>
       </c>
       <c r="N17">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.03</v>
       </c>
       <c r="O17">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>2.5</v>
       </c>
       <c r="P17" s="10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>6.25</v>
       </c>
       <c r="Q17" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v># H-V/Bulk</v>
       </c>
       <c r="U17">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>15</v>
       </c>
       <c r="V17">
@@ -4691,7 +4785,7 @@
         <v>C1MT</v>
       </c>
       <c r="Z17" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>SMT-C1MT</v>
       </c>
       <c r="AB17" t="s">
@@ -4715,7 +4809,7 @@
         <v>128</v>
       </c>
       <c r="AM17">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>15</v>
       </c>
       <c r="AN17">
@@ -4739,7 +4833,7 @@
         <v>HMT</v>
       </c>
       <c r="AS17" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>O1MT-C1MT-HMT</v>
       </c>
       <c r="AU17" t="s">
@@ -4766,7 +4860,7 @@
         <v>178</v>
       </c>
       <c r="BE17">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>15</v>
       </c>
       <c r="BF17">
@@ -4794,7 +4888,7 @@
         <v>0</v>
       </c>
       <c r="BL17">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="BM17" t="str">
@@ -4832,7 +4926,7 @@
     </row>
     <row r="18" spans="2:76" x14ac:dyDescent="0.25">
       <c r="B18">
-        <f t="shared" ref="B18:B20" si="17">B17+1</f>
+        <f t="shared" ref="B18:B20" si="19">B17+1</f>
         <v>16</v>
       </c>
       <c r="C18" t="str">
@@ -4843,52 +4937,53 @@
         <f>MTFSI_LMP_GMX_UniqueMap!M8</f>
         <v>14.007</v>
       </c>
-      <c r="E18">
-        <f>B18</f>
+      <c r="E18" s="15">
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="F18">
+      <c r="F18" s="15">
         <f>MTFSI_LMP_GMX_UniqueMap!J8</f>
         <v>0.17</v>
       </c>
-      <c r="G18">
+      <c r="G18" s="15">
         <f>MTFSI_LMP_GMX_UniqueMap!K8</f>
         <v>3.25</v>
       </c>
-      <c r="H18" t="s">
+      <c r="H18" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="I18" t="s">
+      <c r="I18" s="15" t="s">
         <v>82</v>
       </c>
       <c r="K18" t="s">
         <v>265</v>
       </c>
       <c r="L18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>16</v>
       </c>
-      <c r="M18" s="9" t="s">
-        <v>272</v>
+      <c r="M18" s="9">
+        <f t="shared" si="3"/>
+        <v>16</v>
       </c>
       <c r="N18">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.17</v>
       </c>
       <c r="O18">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>3.25</v>
       </c>
       <c r="P18" s="10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>8.125</v>
       </c>
       <c r="Q18" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v># N-MT/Bulk</v>
       </c>
       <c r="U18">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>16</v>
       </c>
       <c r="V18">
@@ -4908,7 +5003,7 @@
         <v>HV</v>
       </c>
       <c r="Z18" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>C1V-HV</v>
       </c>
       <c r="AB18" t="s">
@@ -4932,7 +5027,7 @@
         <v>129</v>
       </c>
       <c r="AM18">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>16</v>
       </c>
       <c r="AN18">
@@ -4956,7 +5051,7 @@
         <v>FMT</v>
       </c>
       <c r="AS18" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>SMT-C1MT-FMT</v>
       </c>
       <c r="AU18" t="s">
@@ -4980,7 +5075,7 @@
         <v>148</v>
       </c>
       <c r="BE18">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>16</v>
       </c>
       <c r="BF18">
@@ -5008,7 +5103,7 @@
         <v>0</v>
       </c>
       <c r="BL18">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>1.000000000000334E-3</v>
       </c>
       <c r="BM18" t="str">
@@ -5046,7 +5141,7 @@
     </row>
     <row r="19" spans="2:76" x14ac:dyDescent="0.25">
       <c r="B19">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>17</v>
       </c>
       <c r="C19" t="str">
@@ -5057,52 +5152,53 @@
         <f>MTFSI_LMP_GMX_UniqueMap!M7</f>
         <v>15.999000000000001</v>
       </c>
-      <c r="E19">
-        <f>B19</f>
+      <c r="E19" s="15">
+        <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="F19">
+      <c r="F19" s="15">
         <f>MTFSI_LMP_GMX_UniqueMap!J7</f>
         <v>0.14000000000000001</v>
       </c>
-      <c r="G19">
+      <c r="G19" s="15">
         <f>MTFSI_LMP_GMX_UniqueMap!K7</f>
         <v>2.9</v>
       </c>
-      <c r="H19" t="s">
+      <c r="H19" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="I19" t="s">
+      <c r="I19" s="15" t="s">
         <v>83</v>
       </c>
       <c r="K19" t="s">
         <v>265</v>
       </c>
       <c r="L19">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>17</v>
       </c>
-      <c r="M19" s="9" t="s">
-        <v>272</v>
+      <c r="M19" s="9">
+        <f t="shared" si="3"/>
+        <v>17</v>
       </c>
       <c r="N19">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.14000000000000001</v>
       </c>
       <c r="O19">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>2.9</v>
       </c>
       <c r="P19" s="10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>7.25</v>
       </c>
       <c r="Q19" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v># O1-MT/Bulk</v>
       </c>
       <c r="U19">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>17</v>
       </c>
       <c r="V19">
@@ -5122,7 +5218,7 @@
         <v>C2V</v>
       </c>
       <c r="Z19" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>O2V-C2V</v>
       </c>
       <c r="AB19" t="s">
@@ -5146,7 +5242,7 @@
         <v>131</v>
       </c>
       <c r="AM19">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>17</v>
       </c>
       <c r="AN19">
@@ -5170,7 +5266,7 @@
         <v>HMT</v>
       </c>
       <c r="AS19" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>SMT-C1MT-HMT</v>
       </c>
       <c r="AU19" t="s">
@@ -5194,7 +5290,7 @@
         <v>149</v>
       </c>
       <c r="BE19">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>17</v>
       </c>
       <c r="BF19">
@@ -5222,7 +5318,7 @@
         <v>0</v>
       </c>
       <c r="BL19">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>1.000000000000334E-3</v>
       </c>
       <c r="BM19" t="str">
@@ -5260,7 +5356,7 @@
     </row>
     <row r="20" spans="2:76" x14ac:dyDescent="0.25">
       <c r="B20">
-        <f t="shared" si="17"/>
+        <f t="shared" si="19"/>
         <v>18</v>
       </c>
       <c r="C20" t="str">
@@ -5271,52 +5367,53 @@
         <f>VEC_LMP_GMX_UniqueMap!M4</f>
         <v>15.999000000000001</v>
       </c>
-      <c r="E20">
-        <f>B20</f>
+      <c r="E20" s="15">
+        <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="F20">
+      <c r="F20" s="15">
         <f>VEC_LMP_GMX_UniqueMap!J4</f>
         <v>0.14000000000000001</v>
       </c>
-      <c r="G20">
+      <c r="G20" s="15">
         <f>VEC_LMP_GMX_UniqueMap!K4</f>
         <v>2.9</v>
       </c>
-      <c r="H20" t="s">
+      <c r="H20" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="I20" t="s">
+      <c r="I20" s="15" t="s">
         <v>84</v>
       </c>
       <c r="K20" t="s">
         <v>265</v>
       </c>
       <c r="L20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>18</v>
       </c>
-      <c r="M20" s="9" t="s">
-        <v>272</v>
+      <c r="M20" s="9">
+        <f t="shared" si="3"/>
+        <v>18</v>
       </c>
       <c r="N20">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.14000000000000001</v>
       </c>
       <c r="O20">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>2.9</v>
       </c>
       <c r="P20" s="10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>7.25</v>
       </c>
       <c r="Q20" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v># O1-VEC/Bulk</v>
       </c>
       <c r="U20">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>18</v>
       </c>
       <c r="V20">
@@ -5336,7 +5433,7 @@
         <v>O1V</v>
       </c>
       <c r="Z20" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>C2V-O1V</v>
       </c>
       <c r="AB20" t="s">
@@ -5360,7 +5457,7 @@
         <v>114</v>
       </c>
       <c r="AM20">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>18</v>
       </c>
       <c r="AN20">
@@ -5384,7 +5481,7 @@
         <v>HMT</v>
       </c>
       <c r="AS20" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>C2MT-C1MT-HMT</v>
       </c>
       <c r="AU20" t="s">
@@ -5408,7 +5505,7 @@
         <v>170</v>
       </c>
       <c r="BE20">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>18</v>
       </c>
       <c r="BF20">
@@ -5436,7 +5533,7 @@
         <v>0</v>
       </c>
       <c r="BL20">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="BM20" t="str">
@@ -5484,52 +5581,53 @@
         <f>MTFSI_LMP_GMX_UniqueMap!M10</f>
         <v>15.999000000000001</v>
       </c>
-      <c r="E21">
-        <f>B21</f>
+      <c r="E21" s="15">
+        <f t="shared" si="0"/>
         <v>19</v>
       </c>
-      <c r="F21">
+      <c r="F21" s="15">
         <f>MTFSI_LMP_GMX_UniqueMap!J10</f>
         <v>0.21</v>
       </c>
-      <c r="G21">
+      <c r="G21" s="15">
         <f>MTFSI_LMP_GMX_UniqueMap!K10</f>
         <v>2.96</v>
       </c>
-      <c r="H21" t="s">
+      <c r="H21" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="I21" t="s">
+      <c r="I21" s="15" t="s">
         <v>85</v>
       </c>
       <c r="K21" t="s">
         <v>265</v>
       </c>
       <c r="L21">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>19</v>
       </c>
-      <c r="M21" s="9" t="s">
-        <v>272</v>
+      <c r="M21" s="9">
+        <f t="shared" si="3"/>
+        <v>19</v>
       </c>
       <c r="N21">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.21</v>
       </c>
       <c r="O21">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>2.96</v>
       </c>
       <c r="P21" s="10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>7.4</v>
       </c>
       <c r="Q21" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v># O2-MT/Bulk</v>
       </c>
       <c r="U21">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>19</v>
       </c>
       <c r="V21">
@@ -5549,7 +5647,7 @@
         <v>C1V</v>
       </c>
       <c r="Z21" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>O1V-C1V</v>
       </c>
       <c r="AB21" t="s">
@@ -5573,7 +5671,7 @@
         <v>130</v>
       </c>
       <c r="AM21">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>19</v>
       </c>
       <c r="AN21">
@@ -5597,7 +5695,7 @@
         <v>C1MT</v>
       </c>
       <c r="AS21" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>HMT-C1MT-C1MT</v>
       </c>
       <c r="AU21" t="s">
@@ -5621,7 +5719,7 @@
         <v>150</v>
       </c>
       <c r="BE21">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>19</v>
       </c>
       <c r="BF21">
@@ -5649,7 +5747,7 @@
         <v>0</v>
       </c>
       <c r="BL21">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="BM21" t="str">
@@ -5667,15 +5765,15 @@
         <v>1.3</v>
       </c>
       <c r="BS21" s="7">
-        <f t="shared" ref="BS21:BU21" si="18">BS62</f>
+        <f t="shared" ref="BS21:BU21" si="20">BS62</f>
         <v>-0.2</v>
       </c>
       <c r="BT21" s="7">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>0.2</v>
       </c>
       <c r="BU21" s="7">
-        <f t="shared" si="18"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="BV21" s="7" t="s">
@@ -5701,52 +5799,53 @@
         <f>VEC_LMP_GMX_UniqueMap!M5</f>
         <v>15.999000000000001</v>
       </c>
-      <c r="E22">
-        <f>B22</f>
+      <c r="E22" s="15">
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="F22">
+      <c r="F22" s="15">
         <f>VEC_LMP_GMX_UniqueMap!J5</f>
         <v>0.21</v>
       </c>
-      <c r="G22">
+      <c r="G22" s="15">
         <f>VEC_LMP_GMX_UniqueMap!K5</f>
         <v>2.96</v>
       </c>
-      <c r="H22" t="s">
+      <c r="H22" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="I22" t="s">
+      <c r="I22" s="15" t="s">
         <v>86</v>
       </c>
       <c r="K22" t="s">
         <v>265</v>
       </c>
       <c r="L22">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="M22" s="9" t="s">
-        <v>272</v>
+      <c r="M22" s="9">
+        <f t="shared" si="3"/>
+        <v>20</v>
       </c>
       <c r="N22">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.21</v>
       </c>
       <c r="O22">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>2.96</v>
       </c>
       <c r="P22" s="10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>7.4</v>
       </c>
       <c r="Q22" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v># O2-VEC/Bulk</v>
       </c>
       <c r="U22">
-        <f t="shared" si="9"/>
+        <f t="shared" si="11"/>
         <v>20</v>
       </c>
       <c r="V22">
@@ -5766,7 +5865,7 @@
         <v>C1V</v>
       </c>
       <c r="Z22" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>C1V-C1V</v>
       </c>
       <c r="AB22" t="s">
@@ -5790,7 +5889,7 @@
         <v>115</v>
       </c>
       <c r="AM22">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>20</v>
       </c>
       <c r="AN22">
@@ -5814,7 +5913,7 @@
         <v>C2MT</v>
       </c>
       <c r="AS22" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>C1MT-C1MT-C2MT</v>
       </c>
       <c r="AU22" t="s">
@@ -5838,7 +5937,7 @@
         <v>151</v>
       </c>
       <c r="BE22">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>20</v>
       </c>
       <c r="BF22">
@@ -5866,7 +5965,7 @@
         <v>0</v>
       </c>
       <c r="BL22">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="BM22" t="str">
@@ -5884,15 +5983,15 @@
         <v>0</v>
       </c>
       <c r="BS22" s="7">
-        <f t="shared" ref="BS22:BU22" si="19">BS11</f>
+        <f t="shared" ref="BS22:BU22" si="21">BS11</f>
         <v>0</v>
       </c>
       <c r="BT22" s="7">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>0.3</v>
       </c>
       <c r="BU22" s="7">
-        <f t="shared" si="19"/>
+        <f t="shared" si="21"/>
         <v>0</v>
       </c>
       <c r="BV22" s="7" t="s">
@@ -5908,7 +6007,7 @@
     </row>
     <row r="23" spans="2:76" x14ac:dyDescent="0.25">
       <c r="B23">
-        <f t="shared" ref="B23:B24" si="20">B22+1</f>
+        <f t="shared" ref="B23:B24" si="22">B22+1</f>
         <v>21</v>
       </c>
       <c r="C23" t="str">
@@ -5919,48 +6018,49 @@
         <f>MTFSI_LMP_GMX_UniqueMap!M9</f>
         <v>15.999000000000001</v>
       </c>
-      <c r="E23">
-        <f>B23</f>
+      <c r="E23" s="15">
+        <f t="shared" si="0"/>
         <v>21</v>
       </c>
-      <c r="F23">
+      <c r="F23" s="15">
         <f>MTFSI_LMP_GMX_UniqueMap!J9</f>
         <v>0.17</v>
       </c>
-      <c r="G23">
+      <c r="G23" s="15">
         <f>MTFSI_LMP_GMX_UniqueMap!K9</f>
         <v>2.96</v>
       </c>
-      <c r="H23" t="s">
+      <c r="H23" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" s="15" t="s">
         <v>87</v>
       </c>
       <c r="K23" t="s">
         <v>265</v>
       </c>
       <c r="L23">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>21</v>
       </c>
-      <c r="M23" s="9" t="s">
-        <v>272</v>
+      <c r="M23" s="9">
+        <f t="shared" si="3"/>
+        <v>21</v>
       </c>
       <c r="N23">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.17</v>
       </c>
       <c r="O23">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>2.96</v>
       </c>
       <c r="P23" s="10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>7.4</v>
       </c>
       <c r="Q23" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v># O3-MT/Bulk</v>
       </c>
       <c r="AB23" t="s">
@@ -5984,7 +6084,7 @@
         <v>116</v>
       </c>
       <c r="AM23">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>21</v>
       </c>
       <c r="AN23">
@@ -6008,7 +6108,7 @@
         <v>O1MT</v>
       </c>
       <c r="AS23" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>C1MT-C2MT-O1MT</v>
       </c>
       <c r="AU23" t="s">
@@ -6035,7 +6135,7 @@
         <v>177</v>
       </c>
       <c r="BE23">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>21</v>
       </c>
       <c r="BF23">
@@ -6063,7 +6163,7 @@
         <v>0</v>
       </c>
       <c r="BL23">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="BM23" t="str">
@@ -6081,15 +6181,15 @@
         <v>1.7110000000000001</v>
       </c>
       <c r="BS23" s="8">
-        <f t="shared" ref="BS23:BU23" si="21">BS12</f>
+        <f t="shared" ref="BS23:BU23" si="23">BS12</f>
         <v>-0.5</v>
       </c>
       <c r="BT23" s="8">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v>0.66300000000000003</v>
       </c>
       <c r="BU23" s="8">
-        <f t="shared" si="21"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="BV23" s="8" t="s">
@@ -6105,7 +6205,7 @@
     </row>
     <row r="24" spans="2:76" x14ac:dyDescent="0.25">
       <c r="B24">
-        <f t="shared" si="20"/>
+        <f t="shared" si="22"/>
         <v>22</v>
       </c>
       <c r="C24" t="str">
@@ -6116,52 +6216,53 @@
         <f>MTFSI_LMP_GMX_UniqueMap!M11</f>
         <v>32.06</v>
       </c>
-      <c r="E24">
-        <f>B24</f>
+      <c r="E24" s="15">
+        <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="F24">
+      <c r="F24" s="15">
         <f>MTFSI_LMP_GMX_UniqueMap!J11</f>
         <v>0.25</v>
       </c>
-      <c r="G24">
+      <c r="G24" s="15">
         <f>MTFSI_LMP_GMX_UniqueMap!K11</f>
         <v>3.55</v>
       </c>
-      <c r="H24" t="s">
+      <c r="H24" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="I24" t="s">
+      <c r="I24" s="15" t="s">
         <v>88</v>
       </c>
       <c r="K24" t="s">
         <v>265</v>
       </c>
       <c r="L24">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>22</v>
       </c>
-      <c r="M24" s="9" t="s">
-        <v>272</v>
+      <c r="M24" s="9">
+        <f t="shared" si="3"/>
+        <v>22</v>
       </c>
       <c r="N24">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.25</v>
       </c>
       <c r="O24">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>3.55</v>
       </c>
       <c r="P24" s="10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>8.875</v>
       </c>
       <c r="Q24" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v># S-MT/Bulk</v>
       </c>
       <c r="AM24">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>22</v>
       </c>
       <c r="AN24">
@@ -6185,7 +6286,7 @@
         <v>C1MT</v>
       </c>
       <c r="AS24" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>C1MT-C1MT-C1MT</v>
       </c>
       <c r="AU24" t="s">
@@ -6212,7 +6313,7 @@
         <v>178</v>
       </c>
       <c r="BE24">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>22</v>
       </c>
       <c r="BF24">
@@ -6240,7 +6341,7 @@
         <v>0</v>
       </c>
       <c r="BL24">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="BM24" t="str">
@@ -6276,69 +6377,17 @@
         <v>232</v>
       </c>
       <c r="BX24" t="str">
-        <f t="shared" ref="BX24" si="22">BW24</f>
+        <f t="shared" ref="BX24" si="24">BW24</f>
         <v>C1MT-O1MT-C2MT-C1MT</v>
       </c>
     </row>
     <row r="25" spans="2:76" x14ac:dyDescent="0.25">
-      <c r="B25">
-        <v>23</v>
-      </c>
-      <c r="C25" t="str">
-        <f>C7</f>
-        <v>LP</v>
-      </c>
-      <c r="D25">
-        <f>D7</f>
-        <v>6.9409999999999998</v>
-      </c>
-      <c r="E25">
-        <f>B25</f>
-        <v>23</v>
-      </c>
-      <c r="F25">
-        <f>F7</f>
-        <v>0.4</v>
-      </c>
-      <c r="G25">
-        <f>G7</f>
-        <v>1.4</v>
-      </c>
-      <c r="H25" t="str">
-        <f t="shared" ref="H25" si="23">H7</f>
-        <v>#</v>
-      </c>
-      <c r="I25" t="s">
-        <v>274</v>
-      </c>
-      <c r="K25" t="s">
-        <v>265</v>
-      </c>
-      <c r="L25">
-        <f t="shared" si="1"/>
-        <v>23</v>
-      </c>
-      <c r="M25" s="9" t="s">
+      <c r="M25" s="9"/>
+      <c r="AC25" s="16" t="s">
         <v>272</v>
       </c>
-      <c r="N25">
-        <f t="shared" si="2"/>
-        <v>0.4</v>
-      </c>
-      <c r="O25">
-        <f t="shared" si="3"/>
-        <v>1.4</v>
-      </c>
-      <c r="P25" s="10">
-        <f t="shared" si="4"/>
-        <v>3.5</v>
-      </c>
-      <c r="Q25" t="str">
-        <f t="shared" si="5"/>
-        <v># Li-LP/Bulk (Table1: https://pubs.acs.org/doi/10.1021/acs.jpcb.3c05591, Wu-Wick)</v>
-      </c>
       <c r="AM25">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>23</v>
       </c>
       <c r="AN25">
@@ -6362,7 +6411,7 @@
         <v>SMT</v>
       </c>
       <c r="AS25" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>SMT-NMT-SMT</v>
       </c>
       <c r="AU25" t="s">
@@ -6386,7 +6435,7 @@
         <v>154</v>
       </c>
       <c r="BE25">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>23</v>
       </c>
       <c r="BF25">
@@ -6414,7 +6463,7 @@
         <v>0</v>
       </c>
       <c r="BL25">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="BM25" t="str">
@@ -6432,15 +6481,15 @@
         <v>1.3</v>
       </c>
       <c r="BS25" s="7">
-        <f t="shared" ref="BS25:BU26" si="24">BS62</f>
+        <f t="shared" ref="BS25:BU26" si="25">BS62</f>
         <v>-0.2</v>
       </c>
       <c r="BT25" s="7">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>0.2</v>
       </c>
       <c r="BU25" s="7">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>0</v>
       </c>
       <c r="BV25" s="7" t="s">
@@ -6454,8 +6503,9 @@
       </c>
     </row>
     <row r="26" spans="2:76" x14ac:dyDescent="0.25">
+      <c r="M26" s="9"/>
       <c r="AM26">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>24</v>
       </c>
       <c r="AN26">
@@ -6479,7 +6529,7 @@
         <v>C1MT</v>
       </c>
       <c r="AS26" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>C2MT-O1MT-C1MT</v>
       </c>
       <c r="AU26" t="s">
@@ -6503,7 +6553,7 @@
         <v>171</v>
       </c>
       <c r="BE26">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>24</v>
       </c>
       <c r="BF26">
@@ -6531,7 +6581,7 @@
         <v>0</v>
       </c>
       <c r="BL26">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="BM26" t="str">
@@ -6549,15 +6599,15 @@
         <v>-2.06</v>
       </c>
       <c r="BS26" s="7">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>-0.313</v>
       </c>
       <c r="BT26" s="7">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>0.315</v>
       </c>
       <c r="BU26" s="7">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v>0</v>
       </c>
       <c r="BV26" s="7" t="s">
@@ -6571,8 +6621,9 @@
       </c>
     </row>
     <row r="27" spans="2:76" x14ac:dyDescent="0.25">
+      <c r="M27" s="9"/>
       <c r="AM27">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>25</v>
       </c>
       <c r="AN27">
@@ -6596,7 +6647,7 @@
         <v>O3MT</v>
       </c>
       <c r="AS27" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>O3MT-SMT-O3MT</v>
       </c>
       <c r="AU27" t="s">
@@ -6620,7 +6671,7 @@
         <v>155</v>
       </c>
       <c r="BE27">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>25</v>
       </c>
       <c r="BF27">
@@ -6648,7 +6699,7 @@
         <v>0</v>
       </c>
       <c r="BL27">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>-9.9999999999988987E-4</v>
       </c>
       <c r="BM27" t="str">
@@ -6666,15 +6717,15 @@
         <v>0</v>
       </c>
       <c r="BS27" s="7">
-        <f t="shared" ref="BS27:BU27" si="25">BS11</f>
+        <f t="shared" ref="BS27:BU27" si="26">BS11</f>
         <v>0</v>
       </c>
       <c r="BT27" s="7">
-        <f t="shared" si="25"/>
+        <f t="shared" si="26"/>
         <v>0.3</v>
       </c>
       <c r="BU27" s="7">
-        <f t="shared" si="25"/>
+        <f t="shared" si="26"/>
         <v>0</v>
       </c>
       <c r="BV27" s="7" t="s">
@@ -6689,8 +6740,15 @@
       </c>
     </row>
     <row r="28" spans="2:76" x14ac:dyDescent="0.25">
+      <c r="F28" s="20" t="s">
+        <v>273</v>
+      </c>
+      <c r="G28" s="20"/>
+      <c r="H28" s="20"/>
+      <c r="I28" s="20"/>
+      <c r="M28" s="9"/>
       <c r="AM28">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>26</v>
       </c>
       <c r="AN28">
@@ -6714,7 +6772,7 @@
         <v>O2MT</v>
       </c>
       <c r="AS28" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>C1MT-C2MT-O2MT</v>
       </c>
       <c r="AU28" t="s">
@@ -6738,7 +6796,7 @@
         <v>156</v>
       </c>
       <c r="BE28">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>26</v>
       </c>
       <c r="BF28">
@@ -6766,7 +6824,7 @@
         <v>0</v>
       </c>
       <c r="BL28">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="BM28" t="str">
@@ -6784,15 +6842,15 @@
         <v>0</v>
       </c>
       <c r="BS28" s="7">
-        <f t="shared" ref="BS28:BU28" si="26">BS16</f>
+        <f t="shared" ref="BS28:BU28" si="27">BS16</f>
         <v>0</v>
       </c>
       <c r="BT28" s="7">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v>-0.55300000000000005</v>
       </c>
       <c r="BU28" s="7">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v>0</v>
       </c>
       <c r="BV28" s="7" t="s">
@@ -6807,8 +6865,9 @@
       </c>
     </row>
     <row r="29" spans="2:76" x14ac:dyDescent="0.25">
+      <c r="M29" s="9"/>
       <c r="AM29">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>27</v>
       </c>
       <c r="AN29">
@@ -6832,7 +6891,7 @@
         <v>O2MT</v>
       </c>
       <c r="AS29" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>O1MT-C2MT-O2MT</v>
       </c>
       <c r="AU29" t="s">
@@ -6856,7 +6915,7 @@
         <v>157</v>
       </c>
       <c r="BE29">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>27</v>
       </c>
       <c r="BF29">
@@ -6884,7 +6943,7 @@
         <v>0</v>
       </c>
       <c r="BL29">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>4.4408920985006262E-16</v>
       </c>
       <c r="BM29" t="str">
@@ -6902,15 +6961,15 @@
         <v>0</v>
       </c>
       <c r="BS29" s="7">
-        <f t="shared" ref="BS29:BU29" si="27">BS17</f>
+        <f t="shared" ref="BS29:BU29" si="28">BS17</f>
         <v>0</v>
       </c>
       <c r="BT29" s="7">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>0</v>
       </c>
       <c r="BU29" s="7">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v>0</v>
       </c>
       <c r="BV29" s="7" t="s">
@@ -6925,8 +6984,39 @@
       </c>
     </row>
     <row r="30" spans="2:76" x14ac:dyDescent="0.25">
+      <c r="B30" s="17">
+        <v>23</v>
+      </c>
+      <c r="C30" s="17" t="str">
+        <f>C7</f>
+        <v>LP</v>
+      </c>
+      <c r="D30" s="17">
+        <f>D7</f>
+        <v>6.9409999999999998</v>
+      </c>
+      <c r="E30" s="17">
+        <f>B30</f>
+        <v>23</v>
+      </c>
+      <c r="F30" s="17">
+        <f>F7</f>
+        <v>0.4</v>
+      </c>
+      <c r="G30" s="17">
+        <f>G7</f>
+        <v>1.4</v>
+      </c>
+      <c r="H30" s="17" t="str">
+        <f>H7</f>
+        <v>#</v>
+      </c>
+      <c r="I30" s="17" t="s">
+        <v>271</v>
+      </c>
+      <c r="M30" s="9"/>
       <c r="AM30">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>28</v>
       </c>
       <c r="AN30">
@@ -6950,7 +7040,7 @@
         <v>HV</v>
       </c>
       <c r="AS30" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>HV-C1V-HV</v>
       </c>
       <c r="AU30" t="s">
@@ -6974,7 +7064,7 @@
         <v>172</v>
       </c>
       <c r="BE30">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>28</v>
       </c>
       <c r="BF30">
@@ -7002,7 +7092,7 @@
         <v>0</v>
       </c>
       <c r="BL30">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="BM30" t="str">
@@ -7039,8 +7129,37 @@
       </c>
     </row>
     <row r="31" spans="2:76" x14ac:dyDescent="0.25">
+      <c r="B31" s="17" t="s">
+        <v>265</v>
+      </c>
+      <c r="C31" s="17">
+        <f>E30</f>
+        <v>23</v>
+      </c>
+      <c r="D31" s="18">
+        <f>E30</f>
+        <v>23</v>
+      </c>
+      <c r="E31" s="17">
+        <f>F30</f>
+        <v>0.4</v>
+      </c>
+      <c r="F31" s="17">
+        <f>G30</f>
+        <v>1.4</v>
+      </c>
+      <c r="G31" s="19">
+        <f>2.5*F31</f>
+        <v>3.5</v>
+      </c>
+      <c r="H31" s="17" t="str">
+        <f>H30&amp;" "&amp;I30</f>
+        <v># Li-LP/Bulk (Table1: https://pubs.acs.org/doi/10.1021/acs.jpcb.3c05591, Wu-Wick)</v>
+      </c>
+      <c r="I31" s="17"/>
+      <c r="M31" s="9"/>
       <c r="AM31">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>29</v>
       </c>
       <c r="AN31">
@@ -7064,31 +7183,31 @@
         <v>HV</v>
       </c>
       <c r="AS31" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>O1V-C1V-HV</v>
       </c>
       <c r="AU31" t="s">
         <v>260</v>
       </c>
-      <c r="AV31">
+      <c r="AV31" s="16">
         <v>29</v>
       </c>
-      <c r="AW31" cm="1">
+      <c r="AW31" s="16" cm="1">
         <f t="array" ref="AW31">_xlfn.XLOOKUP(AZ31,$AS$3:$AS$37,ROUND(0.119502868*$AO$3:$AO$37,3))</f>
         <v>33</v>
       </c>
-      <c r="AX31" cm="1">
+      <c r="AX31" s="16" cm="1">
         <f t="array" ref="AX31">_xlfn.XLOOKUP(AZ31,$AS$3:$AS$37,ROUND($AN$3:$AN$37,3))</f>
         <v>107.8</v>
       </c>
-      <c r="AY31" t="s">
+      <c r="AY31" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="AZ31" t="s">
+      <c r="AZ31" s="16" t="s">
         <v>158</v>
       </c>
       <c r="BE31">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>29</v>
       </c>
       <c r="BF31">
@@ -7116,7 +7235,7 @@
         <v>0</v>
       </c>
       <c r="BL31">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>-4.4408920985006262E-16</v>
       </c>
       <c r="BM31" t="str">
@@ -7153,8 +7272,9 @@
       </c>
     </row>
     <row r="32" spans="2:76" x14ac:dyDescent="0.25">
+      <c r="M32" s="9"/>
       <c r="AM32">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>30</v>
       </c>
       <c r="AN32">
@@ -7178,7 +7298,7 @@
         <v>C1V</v>
       </c>
       <c r="AS32" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>HV-C1V-C1V</v>
       </c>
       <c r="AU32" t="s">
@@ -7202,7 +7322,7 @@
         <v>173</v>
       </c>
       <c r="BE32">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>30</v>
       </c>
       <c r="BF32">
@@ -7230,7 +7350,7 @@
         <v>0</v>
       </c>
       <c r="BL32">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="BM32" t="str">
@@ -7266,9 +7386,10 @@
         <v>233</v>
       </c>
     </row>
-    <row r="33" spans="39:76" x14ac:dyDescent="0.25">
+    <row r="33" spans="13:76" x14ac:dyDescent="0.25">
+      <c r="M33" s="9"/>
       <c r="AM33">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>31</v>
       </c>
       <c r="AN33">
@@ -7292,7 +7413,7 @@
         <v>O1V</v>
       </c>
       <c r="AS33" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>C1V-C1V-O1V</v>
       </c>
       <c r="AU33" t="s">
@@ -7316,7 +7437,7 @@
         <v>174</v>
       </c>
       <c r="BE33">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>31</v>
       </c>
       <c r="BF33">
@@ -7344,7 +7465,7 @@
         <v>0</v>
       </c>
       <c r="BL33">
-        <f t="shared" si="8"/>
+        <f t="shared" si="10"/>
         <v>-8.8817841970012523E-16</v>
       </c>
       <c r="BM33" t="str">
@@ -7380,9 +7501,10 @@
         <v>234</v>
       </c>
     </row>
-    <row r="34" spans="39:76" x14ac:dyDescent="0.25">
+    <row r="34" spans="13:76" x14ac:dyDescent="0.25">
+      <c r="M34" s="9"/>
       <c r="AM34">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>32</v>
       </c>
       <c r="AN34">
@@ -7406,7 +7528,7 @@
         <v>C1V</v>
       </c>
       <c r="AS34" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>C1V-C1V-C1V</v>
       </c>
       <c r="AU34" t="s">
@@ -7430,7 +7552,7 @@
         <v>159</v>
       </c>
       <c r="BE34">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>32</v>
       </c>
       <c r="BF34">
@@ -7458,7 +7580,7 @@
         <v>0</v>
       </c>
       <c r="BL34">
-        <f t="shared" ref="BL34:BL43" si="28">SUM(BF34:BK34)</f>
+        <f t="shared" ref="BL34:BL43" si="29">SUM(BF34:BK34)</f>
         <v>-4.4408920985006262E-16</v>
       </c>
       <c r="BM34" t="str">
@@ -7494,9 +7616,10 @@
         <v>202</v>
       </c>
     </row>
-    <row r="35" spans="39:76" x14ac:dyDescent="0.25">
+    <row r="35" spans="13:76" x14ac:dyDescent="0.25">
+      <c r="M35" s="9"/>
       <c r="AM35">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>33</v>
       </c>
       <c r="AN35">
@@ -7520,31 +7643,31 @@
         <v>O1V</v>
       </c>
       <c r="AS35" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>O1V-C2V-O1V</v>
       </c>
       <c r="AU35" t="s">
         <v>260</v>
       </c>
-      <c r="AV35">
+      <c r="AV35" s="16">
         <v>33</v>
       </c>
-      <c r="AW35" cm="1">
+      <c r="AW35" s="16" cm="1">
         <f t="array" ref="AW35">_xlfn.XLOOKUP(AZ35,$AS$3:$AS$37,ROUND(0.119502868*$AO$3:$AO$37,3))</f>
         <v>35</v>
       </c>
-      <c r="AX35" cm="1">
+      <c r="AX35" s="16" cm="1">
         <f t="array" ref="AX35">_xlfn.XLOOKUP(AZ35,$AS$3:$AS$37,ROUND($AN$3:$AN$37,3))</f>
         <v>109.5</v>
       </c>
-      <c r="AY35" t="s">
+      <c r="AY35" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="AZ35" t="s">
+      <c r="AZ35" s="16" t="s">
         <v>175</v>
       </c>
       <c r="BE35">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>33</v>
       </c>
       <c r="BF35">
@@ -7572,7 +7695,7 @@
         <v>0</v>
       </c>
       <c r="BL35">
-        <f t="shared" si="28"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="BM35" t="str">
@@ -7590,15 +7713,15 @@
         <v>-2.06</v>
       </c>
       <c r="BS35" s="7">
-        <f t="shared" ref="BS35:BU35" si="29">BS63</f>
+        <f t="shared" ref="BS35:BU35" si="30">BS63</f>
         <v>-0.313</v>
       </c>
       <c r="BT35" s="7">
-        <f t="shared" si="29"/>
+        <f t="shared" si="30"/>
         <v>0.315</v>
       </c>
       <c r="BU35" s="7">
-        <f t="shared" si="29"/>
+        <f t="shared" si="30"/>
         <v>0</v>
       </c>
       <c r="BV35" s="7" t="s">
@@ -7611,9 +7734,10 @@
         <v>245</v>
       </c>
     </row>
-    <row r="36" spans="39:76" x14ac:dyDescent="0.25">
+    <row r="36" spans="13:76" x14ac:dyDescent="0.25">
+      <c r="M36" s="9"/>
       <c r="AM36">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>34</v>
       </c>
       <c r="AN36">
@@ -7637,7 +7761,7 @@
         <v>C2V</v>
       </c>
       <c r="AS36" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>C1V-O1V-C2V</v>
       </c>
       <c r="AU36" t="s">
@@ -7661,7 +7785,7 @@
         <v>160</v>
       </c>
       <c r="BE36">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>34</v>
       </c>
       <c r="BF36">
@@ -7689,7 +7813,7 @@
         <v>0</v>
       </c>
       <c r="BL36">
-        <f t="shared" si="28"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="BM36" t="str">
@@ -7707,15 +7831,15 @@
         <v>0</v>
       </c>
       <c r="BS36" s="7">
-        <f t="shared" ref="BS36:BU36" si="30">BS34</f>
+        <f t="shared" ref="BS36:BU36" si="31">BS34</f>
         <v>0</v>
       </c>
       <c r="BT36" s="7">
-        <f t="shared" si="30"/>
+        <f t="shared" si="31"/>
         <v>-0.1</v>
       </c>
       <c r="BU36" s="7">
-        <f t="shared" si="30"/>
+        <f t="shared" si="31"/>
         <v>0</v>
       </c>
       <c r="BV36" s="7" t="s">
@@ -7729,9 +7853,10 @@
         <v>Same as C2MT-C1MT-C1MT-HMT</v>
       </c>
     </row>
-    <row r="37" spans="39:76" x14ac:dyDescent="0.25">
+    <row r="37" spans="13:76" x14ac:dyDescent="0.25">
+      <c r="M37" s="9"/>
       <c r="AM37">
-        <f t="shared" si="10"/>
+        <f t="shared" si="12"/>
         <v>35</v>
       </c>
       <c r="AN37">
@@ -7755,7 +7880,7 @@
         <v>O2V</v>
       </c>
       <c r="AS37" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="9"/>
         <v>O1V-C2V-O2V</v>
       </c>
       <c r="AU37" t="s">
@@ -7779,7 +7904,7 @@
         <v>161</v>
       </c>
       <c r="BE37">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>35</v>
       </c>
       <c r="BF37">
@@ -7807,7 +7932,7 @@
         <v>0</v>
       </c>
       <c r="BL37">
-        <f t="shared" si="28"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="BM37" t="str">
@@ -7843,7 +7968,8 @@
         <v>205</v>
       </c>
     </row>
-    <row r="38" spans="39:76" x14ac:dyDescent="0.25">
+    <row r="38" spans="13:76" x14ac:dyDescent="0.25">
+      <c r="M38" s="9"/>
       <c r="AU38" t="s">
         <v>260</v>
       </c>
@@ -7865,7 +7991,7 @@
         <v>162</v>
       </c>
       <c r="BE38">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>36</v>
       </c>
       <c r="BF38">
@@ -7893,7 +8019,7 @@
         <v>0</v>
       </c>
       <c r="BL38">
-        <f t="shared" si="28"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="BM38" t="str">
@@ -7929,7 +8055,8 @@
         <v>206</v>
       </c>
     </row>
-    <row r="39" spans="39:76" x14ac:dyDescent="0.25">
+    <row r="39" spans="13:76" x14ac:dyDescent="0.25">
+      <c r="M39" s="9"/>
       <c r="AU39" t="s">
         <v>260</v>
       </c>
@@ -7951,7 +8078,7 @@
         <v>163</v>
       </c>
       <c r="BE39">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>37</v>
       </c>
       <c r="BF39">
@@ -7979,7 +8106,7 @@
         <v>0</v>
       </c>
       <c r="BL39">
-        <f t="shared" si="28"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="BM39" t="str">
@@ -8015,7 +8142,8 @@
         <v>207</v>
       </c>
     </row>
-    <row r="40" spans="39:76" x14ac:dyDescent="0.25">
+    <row r="40" spans="13:76" x14ac:dyDescent="0.25">
+      <c r="M40" s="9"/>
       <c r="AU40" t="s">
         <v>260</v>
       </c>
@@ -8037,7 +8165,7 @@
         <v>164</v>
       </c>
       <c r="BE40">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>38</v>
       </c>
       <c r="BF40">
@@ -8065,7 +8193,7 @@
         <v>0</v>
       </c>
       <c r="BL40">
-        <f t="shared" si="28"/>
+        <f t="shared" si="29"/>
         <v>2.2204460492503131E-16</v>
       </c>
       <c r="BM40" t="str">
@@ -8101,7 +8229,8 @@
         <v>208</v>
       </c>
     </row>
-    <row r="41" spans="39:76" x14ac:dyDescent="0.25">
+    <row r="41" spans="13:76" x14ac:dyDescent="0.25">
+      <c r="M41" s="9"/>
       <c r="AU41" t="s">
         <v>260</v>
       </c>
@@ -8123,7 +8252,7 @@
         <v>165</v>
       </c>
       <c r="BE41">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>39</v>
       </c>
       <c r="BF41">
@@ -8151,7 +8280,7 @@
         <v>0</v>
       </c>
       <c r="BL41">
-        <f t="shared" si="28"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="BM41" t="str">
@@ -8187,9 +8316,10 @@
         <v>235</v>
       </c>
     </row>
-    <row r="42" spans="39:76" x14ac:dyDescent="0.25">
+    <row r="42" spans="13:76" x14ac:dyDescent="0.25">
+      <c r="M42" s="9"/>
       <c r="BE42">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>40</v>
       </c>
       <c r="BF42">
@@ -8217,7 +8347,7 @@
         <v>0</v>
       </c>
       <c r="BL42">
-        <f t="shared" si="28"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="BM42" t="str">
@@ -8235,15 +8365,15 @@
         <v>0</v>
       </c>
       <c r="BS42" s="7">
-        <f t="shared" ref="BS42:BU42" si="31">BS31</f>
+        <f t="shared" ref="BS42:BU42" si="32">BS31</f>
         <v>0</v>
       </c>
       <c r="BT42" s="7">
-        <f t="shared" si="31"/>
+        <f t="shared" si="32"/>
         <v>0.3</v>
       </c>
       <c r="BU42" s="7">
-        <f t="shared" si="31"/>
+        <f t="shared" si="32"/>
         <v>0</v>
       </c>
       <c r="BV42" s="7" t="s">
@@ -8257,9 +8387,10 @@
         <v>Same as C1V-C1V-C1V-HV</v>
       </c>
     </row>
-    <row r="43" spans="39:76" x14ac:dyDescent="0.25">
+    <row r="43" spans="13:76" x14ac:dyDescent="0.25">
+      <c r="M43" s="9"/>
       <c r="BE43">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>41</v>
       </c>
       <c r="BF43">
@@ -8287,7 +8418,7 @@
         <v>0</v>
       </c>
       <c r="BL43">
-        <f t="shared" si="28"/>
+        <f t="shared" si="29"/>
         <v>0</v>
       </c>
       <c r="BM43" t="str">
@@ -8305,15 +8436,15 @@
         <v>0</v>
       </c>
       <c r="BS43" s="7">
-        <f t="shared" ref="BS43:BU43" si="32">BS39</f>
+        <f t="shared" ref="BS43:BU43" si="33">BS39</f>
         <v>0</v>
       </c>
       <c r="BT43" s="7">
-        <f t="shared" si="32"/>
+        <f t="shared" si="33"/>
         <v>0.3</v>
       </c>
       <c r="BU43" s="7">
-        <f t="shared" si="32"/>
+        <f t="shared" si="33"/>
         <v>0</v>
       </c>
       <c r="BV43" s="7" t="s">
@@ -8327,7 +8458,8 @@
         <v>Same as HMT-C1MT-C1MT-HMT</v>
       </c>
     </row>
-    <row r="44" spans="39:76" x14ac:dyDescent="0.25">
+    <row r="44" spans="13:76" x14ac:dyDescent="0.25">
+      <c r="M44" s="9"/>
       <c r="BP44" t="s">
         <v>264</v>
       </c>
@@ -8357,7 +8489,8 @@
         <v>211</v>
       </c>
     </row>
-    <row r="45" spans="39:76" x14ac:dyDescent="0.25">
+    <row r="45" spans="13:76" x14ac:dyDescent="0.25">
+      <c r="M45" s="9"/>
       <c r="BP45" t="s">
         <v>264</v>
       </c>
@@ -8387,7 +8520,8 @@
         <v>236</v>
       </c>
     </row>
-    <row r="46" spans="39:76" x14ac:dyDescent="0.25">
+    <row r="46" spans="13:76" x14ac:dyDescent="0.25">
+      <c r="M46" s="9"/>
       <c r="BP46" t="s">
         <v>264</v>
       </c>
@@ -8417,7 +8551,8 @@
         <v>237</v>
       </c>
     </row>
-    <row r="47" spans="39:76" x14ac:dyDescent="0.25">
+    <row r="47" spans="13:76" x14ac:dyDescent="0.25">
+      <c r="M47" s="9"/>
       <c r="BP47" t="s">
         <v>264</v>
       </c>
@@ -8447,7 +8582,8 @@
         <v>212</v>
       </c>
     </row>
-    <row r="48" spans="39:76" x14ac:dyDescent="0.25">
+    <row r="48" spans="13:76" x14ac:dyDescent="0.25">
+      <c r="M48" s="9"/>
       <c r="BP48" t="s">
         <v>264</v>
       </c>
@@ -8739,6 +8875,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="F28:I28"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
updated atom types list
</commit_message>
<xml_diff>
--- a/atomtypes_charges/All_AtomandTopoTypes.xlsx
+++ b/atomtypes_charges/All_AtomandTopoTypes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ornl-my.sharepoint.com/personal/vm5_ornl_gov/Documents/Projects/SingleIonConductors_WithSurface/SIC_Atomistic/atomtypes_charges/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1796" documentId="11_F25DC773A252ABDACC1048D7219A55725ADE5902" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4D6F6D3B-F8D1-417F-82D6-AB193D1992EE}"/>
+  <xr:revisionPtr revIDLastSave="1800" documentId="11_F25DC773A252ABDACC1048D7219A55725ADE5902" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{92BEC085-C45D-4FB8-8205-5B1A81CC6A58}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="All_Unique_Types" sheetId="4" r:id="rId1"/>
@@ -332,12 +332,6 @@
     <t>F-MT/Bulk</t>
   </si>
   <si>
-    <t>H-M/Bulk</t>
-  </si>
-  <si>
-    <t>H-V/Bulk</t>
-  </si>
-  <si>
     <t>N-MT/Bulk</t>
   </si>
   <si>
@@ -348,9 +342,6 @@
   </si>
   <si>
     <t>O2-MT/Bulk</t>
-  </si>
-  <si>
-    <t>O2-VEC/Bulk</t>
   </si>
   <si>
     <t>O3-MT/Bulk</t>
@@ -942,6 +933,15 @@
   <si>
     <t>sigma (Angstrom)</t>
   </si>
+  <si>
+    <t>H-MT/Bulk</t>
+  </si>
+  <si>
+    <t>H-VEC/Bulk</t>
+  </si>
+  <si>
+    <t>O2-VEC/Bulk</t>
+  </si>
 </sst>
 </file>
 
@@ -1104,6 +1104,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1417,31 +1421,31 @@
   <sheetData>
     <row r="1" spans="1:76" ht="120" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="H1" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>104</v>
-      </c>
       <c r="K1" s="1" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="L1" s="1"/>
       <c r="M1" s="1"/>
@@ -1453,52 +1457,52 @@
       <c r="S1" s="1"/>
       <c r="T1" s="1"/>
       <c r="U1" s="1" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="AA1" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="AE1" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="AF1" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="AM1" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="AT1" t="s">
+        <v>130</v>
+      </c>
+      <c r="AV1" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="AX1" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="AY1" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="BE1" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="BQ1" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="BS1" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="BT1" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="BU1" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="BV1" s="1" t="s">
         <v>220</v>
-      </c>
-      <c r="AF1" s="1" t="s">
-        <v>219</v>
-      </c>
-      <c r="AM1" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="AT1" t="s">
-        <v>133</v>
-      </c>
-      <c r="AV1" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="AX1" s="1" t="s">
-        <v>217</v>
-      </c>
-      <c r="AY1" s="1" t="s">
-        <v>218</v>
-      </c>
-      <c r="BE1" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="BQ1" s="1" t="s">
-        <v>261</v>
-      </c>
-      <c r="BS1" s="1" t="s">
-        <v>224</v>
-      </c>
-      <c r="BT1" s="1" t="s">
-        <v>225</v>
-      </c>
-      <c r="BU1" s="1" t="s">
-        <v>222</v>
-      </c>
-      <c r="BV1" s="1" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="2" spans="1:76" x14ac:dyDescent="0.25">
@@ -1515,13 +1519,13 @@
         <v>18</v>
       </c>
       <c r="E2" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="F2" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="G2" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="H2" t="s">
         <v>68</v>
@@ -1530,61 +1534,61 @@
         <v>67</v>
       </c>
       <c r="K2" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="L2" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="M2" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="N2" t="s">
+        <v>264</v>
+      </c>
+      <c r="O2" t="s">
+        <v>273</v>
+      </c>
+      <c r="P2" t="s">
+        <v>271</v>
+      </c>
+      <c r="Q2" t="s">
         <v>267</v>
-      </c>
-      <c r="O2" t="s">
-        <v>276</v>
-      </c>
-      <c r="P2" t="s">
-        <v>274</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>270</v>
       </c>
       <c r="U2" t="s">
         <v>68</v>
       </c>
       <c r="V2" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="W2" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="X2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="Y2" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="Z2" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="AB2" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="AC2" s="1" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="AD2" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="AE2" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="AF2" t="s">
         <v>68</v>
       </c>
       <c r="AG2" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="AM2" t="s">
         <v>68</v>
@@ -1605,19 +1609,19 @@
         <v>8</v>
       </c>
       <c r="AS2" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="AU2" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="AV2" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="AW2" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="AX2" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="AY2" t="s">
         <v>68</v>
@@ -1653,28 +1657,28 @@
         <v>c5 (gmx)</v>
       </c>
       <c r="BL2" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="BM2" t="s">
         <v>17</v>
       </c>
       <c r="BP2" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="BQ2" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="BR2" t="s">
+        <v>244</v>
+      </c>
+      <c r="BS2" t="s">
+        <v>245</v>
+      </c>
+      <c r="BT2" t="s">
+        <v>246</v>
+      </c>
+      <c r="BU2" t="s">
         <v>247</v>
-      </c>
-      <c r="BS2" t="s">
-        <v>248</v>
-      </c>
-      <c r="BT2" t="s">
-        <v>249</v>
-      </c>
-      <c r="BU2" t="s">
-        <v>250</v>
       </c>
       <c r="BV2" t="s">
         <v>68</v>
@@ -1707,10 +1711,10 @@
         <v>68</v>
       </c>
       <c r="I3" s="11" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="K3" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="L3">
         <f>E3</f>
@@ -1760,7 +1764,7 @@
         <v>O1P-C1P</v>
       </c>
       <c r="AB3" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="AC3">
         <v>1</v>
@@ -1777,7 +1781,7 @@
         <v>68</v>
       </c>
       <c r="AG3" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="AM3">
         <v>1</v>
@@ -1807,7 +1811,7 @@
         <v>C1P-O1P-C1P</v>
       </c>
       <c r="AU3" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="AV3">
         <v>1</v>
@@ -1824,7 +1828,7 @@
         <v>68</v>
       </c>
       <c r="AZ3" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="BE3">
         <v>1</v>
@@ -1862,7 +1866,7 @@
         <v>C1P-C1P-O1P-C1P</v>
       </c>
       <c r="BP3" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ3">
         <v>1</v>
@@ -1887,7 +1891,7 @@
         <v>68</v>
       </c>
       <c r="BW3" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
     </row>
     <row r="4" spans="1:76" x14ac:dyDescent="0.25">
@@ -1922,7 +1926,7 @@
         <v>69</v>
       </c>
       <c r="K4" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="L4">
         <f t="shared" ref="L4:L24" si="2">E4</f>
@@ -1973,7 +1977,7 @@
         <v>C1P-C1P</v>
       </c>
       <c r="AB4" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="AC4" s="16">
         <v>2</v>
@@ -1990,7 +1994,7 @@
         <v>68</v>
       </c>
       <c r="AG4" s="16" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="AH4" s="16"/>
       <c r="AM4">
@@ -2022,7 +2026,7 @@
         <v>O1P-C1P-C1P</v>
       </c>
       <c r="AU4" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="AV4">
         <v>2</v>
@@ -2039,7 +2043,7 @@
         <v>68</v>
       </c>
       <c r="AZ4" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="BE4">
         <f>BE3+1</f>
@@ -2078,7 +2082,7 @@
         <v>HP-C1P-C1P-HP</v>
       </c>
       <c r="BP4" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ4">
         <v>2</v>
@@ -2103,7 +2107,7 @@
         <v>68</v>
       </c>
       <c r="BW4" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="5" spans="1:76" x14ac:dyDescent="0.25">
@@ -2138,7 +2142,7 @@
         <v>70</v>
       </c>
       <c r="K5" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="L5">
         <f t="shared" si="2"/>
@@ -2189,7 +2193,7 @@
         <v>HP-C1P</v>
       </c>
       <c r="AB5" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="AC5">
         <v>3</v>
@@ -2206,7 +2210,7 @@
         <v>68</v>
       </c>
       <c r="AG5" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="AM5">
         <f t="shared" ref="AM5:AM37" si="12">AM4+1</f>
@@ -2237,7 +2241,7 @@
         <v>O1P-C1P-HP</v>
       </c>
       <c r="AU5" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="AV5">
         <v>3</v>
@@ -2254,7 +2258,7 @@
         <v>68</v>
       </c>
       <c r="AZ5" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="BE5">
         <f t="shared" ref="BE5:BE43" si="13">BE4+1</f>
@@ -2293,7 +2297,7 @@
         <v>HP-C1P-C1P-O1P</v>
       </c>
       <c r="BP5" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ5">
         <v>3</v>
@@ -2318,7 +2322,7 @@
         <v>68</v>
       </c>
       <c r="BW5" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
     </row>
     <row r="6" spans="1:76" x14ac:dyDescent="0.25">
@@ -2353,7 +2357,7 @@
         <v>71</v>
       </c>
       <c r="K6" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="L6">
         <f t="shared" si="2"/>
@@ -2404,7 +2408,7 @@
         <v>C1C-O1C</v>
       </c>
       <c r="AB6" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="AC6">
         <v>4</v>
@@ -2421,7 +2425,7 @@
         <v>68</v>
       </c>
       <c r="AG6" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="AM6">
         <f t="shared" si="12"/>
@@ -2452,7 +2456,7 @@
         <v>C1P-C1P-HP</v>
       </c>
       <c r="AU6" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="AV6" s="16">
         <v>4</v>
@@ -2469,7 +2473,7 @@
         <v>68</v>
       </c>
       <c r="AZ6" s="16" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="BE6">
         <f t="shared" si="13"/>
@@ -2508,7 +2512,7 @@
         <v>HP-C1P-O1P-C1P</v>
       </c>
       <c r="BP6" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ6">
         <v>4</v>
@@ -2533,7 +2537,7 @@
         <v>68</v>
       </c>
       <c r="BW6" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="7" spans="1:76" x14ac:dyDescent="0.25">
@@ -2542,7 +2546,7 @@
         <v>5</v>
       </c>
       <c r="C7" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="D7">
         <v>6.9409999999999998</v>
@@ -2561,10 +2565,10 @@
         <v>68</v>
       </c>
       <c r="I7" s="13" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="K7" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="L7">
         <f t="shared" si="2"/>
@@ -2615,7 +2619,7 @@
         <v>O2C-C1C</v>
       </c>
       <c r="AB7" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="AC7">
         <v>5</v>
@@ -2632,7 +2636,7 @@
         <v>68</v>
       </c>
       <c r="AG7" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="AM7">
         <f t="shared" si="12"/>
@@ -2663,7 +2667,7 @@
         <v>HP-C1P-HP</v>
       </c>
       <c r="AU7" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="AV7">
         <v>5</v>
@@ -2680,7 +2684,7 @@
         <v>68</v>
       </c>
       <c r="AZ7" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="BE7">
         <f t="shared" si="13"/>
@@ -2719,7 +2723,7 @@
         <v>O1P-C1P-C1P-O1P</v>
       </c>
       <c r="BP7" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ7">
         <v>5</v>
@@ -2744,7 +2748,7 @@
         <v>68</v>
       </c>
       <c r="BW7" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
     </row>
     <row r="8" spans="1:76" x14ac:dyDescent="0.25">
@@ -2779,7 +2783,7 @@
         <v>72</v>
       </c>
       <c r="K8" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="L8">
         <f t="shared" si="2"/>
@@ -2833,7 +2837,7 @@
         <v>C1MT-HMT</v>
       </c>
       <c r="AB8" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="AC8">
         <v>6</v>
@@ -2850,7 +2854,7 @@
         <v>68</v>
       </c>
       <c r="AG8" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="AM8">
         <f t="shared" si="12"/>
@@ -2881,7 +2885,7 @@
         <v>O1C-C1C-O2C</v>
       </c>
       <c r="AU8" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="AV8">
         <v>6</v>
@@ -2898,7 +2902,7 @@
         <v>68</v>
       </c>
       <c r="AZ8" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="BE8">
         <f t="shared" si="13"/>
@@ -2937,7 +2941,7 @@
         <v>C2MT-C1MT-C1MT-HMT</v>
       </c>
       <c r="BP8" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ8">
         <v>6</v>
@@ -2962,10 +2966,10 @@
         <v>68</v>
       </c>
       <c r="BW8" s="7" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="BX8" s="7" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
     </row>
     <row r="9" spans="1:76" x14ac:dyDescent="0.25">
@@ -3000,7 +3004,7 @@
         <v>73</v>
       </c>
       <c r="K9" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="L9">
         <f t="shared" si="2"/>
@@ -3051,7 +3055,7 @@
         <v>O2MT-C2MT</v>
       </c>
       <c r="AB9" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="AC9" s="7">
         <v>7</v>
@@ -3068,7 +3072,7 @@
         <v>68</v>
       </c>
       <c r="AG9" s="7" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="AH9" s="7" t="str">
         <f>"Same as "&amp;AG8</f>
@@ -3103,7 +3107,7 @@
         <v>O2C-C1C-O2C</v>
       </c>
       <c r="AU9" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="AV9">
         <v>7</v>
@@ -3120,7 +3124,7 @@
         <v>68</v>
       </c>
       <c r="AZ9" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="BE9">
         <f t="shared" si="13"/>
@@ -3159,7 +3163,7 @@
         <v>C1MT-SMT-NMT-SMT</v>
       </c>
       <c r="BP9" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ9">
         <v>7</v>
@@ -3184,10 +3188,10 @@
         <v>68</v>
       </c>
       <c r="BW9" s="7" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="BX9" s="7" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
     </row>
     <row r="10" spans="1:76" x14ac:dyDescent="0.25">
@@ -3222,7 +3226,7 @@
         <v>74</v>
       </c>
       <c r="K10" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="L10">
         <f t="shared" si="2"/>
@@ -3273,7 +3277,7 @@
         <v>O1MT-C2MT</v>
       </c>
       <c r="AB10" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="AC10">
         <v>8</v>
@@ -3290,7 +3294,7 @@
         <v>68</v>
       </c>
       <c r="AG10" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="AM10">
         <f t="shared" si="12"/>
@@ -3321,7 +3325,7 @@
         <v>C1MT-SMT-NMT</v>
       </c>
       <c r="AU10" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="AV10">
         <v>8</v>
@@ -3338,7 +3342,7 @@
         <v>68</v>
       </c>
       <c r="AZ10" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="BE10">
         <f t="shared" si="13"/>
@@ -3377,7 +3381,7 @@
         <v>C1MT-C1MT-C1MT-HMT</v>
       </c>
       <c r="BP10" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ10">
         <v>8</v>
@@ -3402,10 +3406,10 @@
         <v>68</v>
       </c>
       <c r="BW10" s="7" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="BX10" s="7" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
     </row>
     <row r="11" spans="1:76" x14ac:dyDescent="0.25">
@@ -3440,7 +3444,7 @@
         <v>75</v>
       </c>
       <c r="K11" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="L11">
         <f t="shared" si="2"/>
@@ -3491,7 +3495,7 @@
         <v>FMT-C1MT</v>
       </c>
       <c r="AB11" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="AC11">
         <v>9</v>
@@ -3508,7 +3512,7 @@
         <v>68</v>
       </c>
       <c r="AG11" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="AM11">
         <f t="shared" si="12"/>
@@ -3539,7 +3543,7 @@
         <v>NMT-SMT-O3MT</v>
       </c>
       <c r="AU11" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="AV11">
         <v>9</v>
@@ -3556,10 +3560,10 @@
         <v>68</v>
       </c>
       <c r="AZ11" s="7" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="BA11" s="7" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="BE11">
         <f t="shared" si="13"/>
@@ -3598,7 +3602,7 @@
         <v>C1MT-C1MT-C1MT-O1MT</v>
       </c>
       <c r="BP11" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ11">
         <v>9</v>
@@ -3623,7 +3627,7 @@
         <v>68</v>
       </c>
       <c r="BW11" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
     </row>
     <row r="12" spans="1:76" x14ac:dyDescent="0.25">
@@ -3657,7 +3661,7 @@
         <v>76</v>
       </c>
       <c r="K12" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="L12">
         <f t="shared" si="2"/>
@@ -3708,7 +3712,7 @@
         <v>C1MT-O1MT</v>
       </c>
       <c r="AB12" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="AC12" s="16">
         <v>10</v>
@@ -3725,7 +3729,7 @@
         <v>68</v>
       </c>
       <c r="AG12" s="16" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="AM12">
         <f t="shared" si="12"/>
@@ -3756,7 +3760,7 @@
         <v>HMT-C1MT-HMT</v>
       </c>
       <c r="AU12" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="AV12">
         <v>10</v>
@@ -3773,7 +3777,7 @@
         <v>68</v>
       </c>
       <c r="AZ12" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="BE12">
         <f t="shared" si="13"/>
@@ -3812,7 +3816,7 @@
         <v>C1MT-C1MT-O1MT-C2MT</v>
       </c>
       <c r="BP12" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ12">
         <v>10</v>
@@ -3837,7 +3841,7 @@
         <v>68</v>
       </c>
       <c r="BW12" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
     </row>
     <row r="13" spans="1:76" x14ac:dyDescent="0.25">
@@ -3871,7 +3875,7 @@
         <v>77</v>
       </c>
       <c r="K13" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="L13">
         <f t="shared" si="2"/>
@@ -3922,7 +3926,7 @@
         <v>O3MT-SMT</v>
       </c>
       <c r="AB13" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="AC13">
         <v>11</v>
@@ -3939,7 +3943,7 @@
         <v>68</v>
       </c>
       <c r="AG13" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="AM13">
         <f t="shared" si="12"/>
@@ -3970,7 +3974,7 @@
         <v>C1MT-C1MT-SMT</v>
       </c>
       <c r="AU13" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="AV13" s="16">
         <v>11</v>
@@ -3987,7 +3991,7 @@
         <v>68</v>
       </c>
       <c r="AZ13" s="16" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="BE13">
         <f t="shared" si="13"/>
@@ -4026,7 +4030,7 @@
         <v>C1MT-O1MT-C2MT-C1MT</v>
       </c>
       <c r="BP13" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ13">
         <v>11</v>
@@ -4051,7 +4055,7 @@
         <v>68</v>
       </c>
       <c r="BW13" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
     </row>
     <row r="14" spans="1:76" x14ac:dyDescent="0.25">
@@ -4085,7 +4089,7 @@
         <v>78</v>
       </c>
       <c r="K14" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="L14">
         <f t="shared" si="2"/>
@@ -4136,7 +4140,7 @@
         <v>C2MT-C1MT</v>
       </c>
       <c r="AB14" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="AC14">
         <v>12</v>
@@ -4153,7 +4157,7 @@
         <v>68</v>
       </c>
       <c r="AG14" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="AM14">
         <f t="shared" si="12"/>
@@ -4184,7 +4188,7 @@
         <v>C1MT-SMT-O3MT</v>
       </c>
       <c r="AU14" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="AV14">
         <v>12</v>
@@ -4201,7 +4205,7 @@
         <v>68</v>
       </c>
       <c r="AZ14" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="BE14">
         <f t="shared" si="13"/>
@@ -4240,7 +4244,7 @@
         <v>C1MT-O1MT-C2MT-O2MT</v>
       </c>
       <c r="BP14" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ14">
         <v>12</v>
@@ -4265,10 +4269,10 @@
         <v>68</v>
       </c>
       <c r="BW14" s="7" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="BX14" s="7" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
     </row>
     <row r="15" spans="1:76" x14ac:dyDescent="0.25">
@@ -4302,7 +4306,7 @@
         <v>79</v>
       </c>
       <c r="K15" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="L15">
         <f t="shared" si="2"/>
@@ -4353,7 +4357,7 @@
         <v>C1MT-C1MT</v>
       </c>
       <c r="AB15" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="AC15">
         <v>13</v>
@@ -4370,7 +4374,7 @@
         <v>68</v>
       </c>
       <c r="AG15" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="AM15">
         <f t="shared" si="12"/>
@@ -4401,7 +4405,7 @@
         <v>FMT-C1MT-FMT</v>
       </c>
       <c r="AU15" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="AV15">
         <v>13</v>
@@ -4418,7 +4422,7 @@
         <v>68</v>
       </c>
       <c r="AZ15" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="BE15">
         <f t="shared" si="13"/>
@@ -4457,7 +4461,7 @@
         <v>FMT-C1MT-SMT-NMT</v>
       </c>
       <c r="BP15" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ15">
         <v>13</v>
@@ -4482,7 +4486,7 @@
         <v>68</v>
       </c>
       <c r="BW15" s="7" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="BX15" s="7" t="str">
         <f>"Same as "&amp;BW11</f>
@@ -4517,10 +4521,10 @@
         <v>68</v>
       </c>
       <c r="I16" s="15" t="s">
-        <v>80</v>
+        <v>274</v>
       </c>
       <c r="K16" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="L16">
         <f t="shared" si="2"/>
@@ -4544,7 +4548,7 @@
       </c>
       <c r="Q16" t="str">
         <f t="shared" si="7"/>
-        <v># H-M/Bulk</v>
+        <v># H-MT/Bulk</v>
       </c>
       <c r="U16">
         <f t="shared" si="11"/>
@@ -4571,7 +4575,7 @@
         <v>NMT-SMT</v>
       </c>
       <c r="AB16" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="AC16" s="16">
         <v>14</v>
@@ -4588,7 +4592,7 @@
         <v>68</v>
       </c>
       <c r="AG16" s="16" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="AM16">
         <f t="shared" si="12"/>
@@ -4619,7 +4623,7 @@
         <v>O1MT-C1MT-C1MT</v>
       </c>
       <c r="AU16" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="AV16">
         <v>14</v>
@@ -4636,10 +4640,10 @@
         <v>68</v>
       </c>
       <c r="AZ16" s="7" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="BA16" s="7" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="BE16">
         <f t="shared" si="13"/>
@@ -4678,7 +4682,7 @@
         <v>FMT-C1MT-SMT-O3MT</v>
       </c>
       <c r="BP16" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ16">
         <v>14</v>
@@ -4703,7 +4707,7 @@
         <v>68</v>
       </c>
       <c r="BW16" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
     </row>
     <row r="17" spans="2:76" x14ac:dyDescent="0.25">
@@ -4735,10 +4739,10 @@
         <v>68</v>
       </c>
       <c r="I17" s="15" t="s">
-        <v>81</v>
+        <v>275</v>
       </c>
       <c r="K17" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="L17">
         <f t="shared" si="2"/>
@@ -4762,7 +4766,7 @@
       </c>
       <c r="Q17" t="str">
         <f t="shared" si="7"/>
-        <v># H-V/Bulk</v>
+        <v># H-VEC/Bulk</v>
       </c>
       <c r="U17">
         <f t="shared" si="11"/>
@@ -4789,7 +4793,7 @@
         <v>SMT-C1MT</v>
       </c>
       <c r="AB17" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="AC17">
         <v>15</v>
@@ -4806,7 +4810,7 @@
         <v>68</v>
       </c>
       <c r="AG17" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="AM17">
         <f t="shared" si="12"/>
@@ -4837,7 +4841,7 @@
         <v>O1MT-C1MT-HMT</v>
       </c>
       <c r="AU17" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="AV17">
         <v>15</v>
@@ -4854,10 +4858,10 @@
         <v>68</v>
       </c>
       <c r="AZ17" s="7" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="BA17" s="7" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="BE17">
         <f t="shared" si="13"/>
@@ -4896,7 +4900,7 @@
         <v>HMT-C1MT-C1MT-C2MT</v>
       </c>
       <c r="BP17" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ17">
         <v>15</v>
@@ -4921,7 +4925,7 @@
         <v>68</v>
       </c>
       <c r="BW17" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
     </row>
     <row r="18" spans="2:76" x14ac:dyDescent="0.25">
@@ -4953,10 +4957,10 @@
         <v>68</v>
       </c>
       <c r="I18" s="15" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="K18" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="L18">
         <f t="shared" si="2"/>
@@ -5007,7 +5011,7 @@
         <v>C1V-HV</v>
       </c>
       <c r="AB18" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="AC18">
         <v>16</v>
@@ -5024,7 +5028,7 @@
         <v>68</v>
       </c>
       <c r="AG18" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="AM18">
         <f t="shared" si="12"/>
@@ -5055,7 +5059,7 @@
         <v>SMT-C1MT-FMT</v>
       </c>
       <c r="AU18" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="AV18">
         <v>16</v>
@@ -5072,7 +5076,7 @@
         <v>68</v>
       </c>
       <c r="AZ18" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="BE18">
         <f t="shared" si="13"/>
@@ -5111,7 +5115,7 @@
         <v>HMT-C1MT-C1MT-C1MT</v>
       </c>
       <c r="BP18" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ18">
         <v>16</v>
@@ -5136,7 +5140,7 @@
         <v>68</v>
       </c>
       <c r="BW18" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
     </row>
     <row r="19" spans="2:76" x14ac:dyDescent="0.25">
@@ -5168,10 +5172,10 @@
         <v>68</v>
       </c>
       <c r="I19" s="15" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="K19" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="L19">
         <f t="shared" si="2"/>
@@ -5222,7 +5226,7 @@
         <v>O2V-C2V</v>
       </c>
       <c r="AB19" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="AC19">
         <v>17</v>
@@ -5239,7 +5243,7 @@
         <v>68</v>
       </c>
       <c r="AG19" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="AM19">
         <f t="shared" si="12"/>
@@ -5270,7 +5274,7 @@
         <v>SMT-C1MT-HMT</v>
       </c>
       <c r="AU19" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="AV19">
         <v>17</v>
@@ -5287,7 +5291,7 @@
         <v>68</v>
       </c>
       <c r="AZ19" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="BE19">
         <f t="shared" si="13"/>
@@ -5326,7 +5330,7 @@
         <v>HMT-C1MT-C1MT-HMT</v>
       </c>
       <c r="BP19" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ19">
         <v>17</v>
@@ -5351,7 +5355,7 @@
         <v>68</v>
       </c>
       <c r="BW19" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
     </row>
     <row r="20" spans="2:76" x14ac:dyDescent="0.25">
@@ -5383,10 +5387,10 @@
         <v>68</v>
       </c>
       <c r="I20" s="15" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="K20" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="L20">
         <f t="shared" si="2"/>
@@ -5437,7 +5441,7 @@
         <v>C2V-O1V</v>
       </c>
       <c r="AB20" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="AC20">
         <v>18</v>
@@ -5454,7 +5458,7 @@
         <v>68</v>
       </c>
       <c r="AG20" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="AM20">
         <f t="shared" si="12"/>
@@ -5485,7 +5489,7 @@
         <v>C2MT-C1MT-HMT</v>
       </c>
       <c r="AU20" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="AV20">
         <v>18</v>
@@ -5502,7 +5506,7 @@
         <v>68</v>
       </c>
       <c r="AZ20" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="BE20">
         <f t="shared" si="13"/>
@@ -5541,7 +5545,7 @@
         <v>HMT-C1MT-C1MT-O1MT</v>
       </c>
       <c r="BP20" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ20">
         <v>18</v>
@@ -5566,7 +5570,7 @@
         <v>68</v>
       </c>
       <c r="BW20" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
     </row>
     <row r="21" spans="2:76" x14ac:dyDescent="0.25">
@@ -5597,10 +5601,10 @@
         <v>68</v>
       </c>
       <c r="I21" s="15" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="K21" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="L21">
         <f t="shared" si="2"/>
@@ -5651,7 +5655,7 @@
         <v>O1V-C1V</v>
       </c>
       <c r="AB21" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="AC21">
         <v>19</v>
@@ -5668,7 +5672,7 @@
         <v>68</v>
       </c>
       <c r="AG21" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="AM21">
         <f t="shared" si="12"/>
@@ -5699,7 +5703,7 @@
         <v>HMT-C1MT-C1MT</v>
       </c>
       <c r="AU21" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="AV21">
         <v>19</v>
@@ -5716,7 +5720,7 @@
         <v>68</v>
       </c>
       <c r="AZ21" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="BE21">
         <f t="shared" si="13"/>
@@ -5755,7 +5759,7 @@
         <v>HMT-C1MT-O1MT-C2MT</v>
       </c>
       <c r="BP21" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ21">
         <v>19</v>
@@ -5780,10 +5784,10 @@
         <v>68</v>
       </c>
       <c r="BW21" s="7" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="BX21" s="7" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
     </row>
     <row r="22" spans="2:76" x14ac:dyDescent="0.25">
@@ -5815,10 +5819,10 @@
         <v>68</v>
       </c>
       <c r="I22" s="15" t="s">
-        <v>86</v>
+        <v>276</v>
       </c>
       <c r="K22" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="L22">
         <f t="shared" si="2"/>
@@ -5869,7 +5873,7 @@
         <v>C1V-C1V</v>
       </c>
       <c r="AB22" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="AC22">
         <v>20</v>
@@ -5886,7 +5890,7 @@
         <v>68</v>
       </c>
       <c r="AG22" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="AM22">
         <f t="shared" si="12"/>
@@ -5917,7 +5921,7 @@
         <v>C1MT-C1MT-C2MT</v>
       </c>
       <c r="AU22" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="AV22">
         <v>20</v>
@@ -5934,7 +5938,7 @@
         <v>68</v>
       </c>
       <c r="AZ22" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="BE22">
         <f t="shared" si="13"/>
@@ -5973,7 +5977,7 @@
         <v>NMT-SMT-C1MT-C1MT</v>
       </c>
       <c r="BP22" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ22">
         <v>20</v>
@@ -5998,7 +6002,7 @@
         <v>68</v>
       </c>
       <c r="BW22" s="7" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="BX22" s="7" t="str">
         <f>"Same as "&amp;BW11</f>
@@ -6034,10 +6038,10 @@
         <v>68</v>
       </c>
       <c r="I23" s="15" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="K23" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="L23">
         <f t="shared" si="2"/>
@@ -6064,7 +6068,7 @@
         <v># O3-MT/Bulk</v>
       </c>
       <c r="AB23" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="AC23">
         <v>21</v>
@@ -6081,7 +6085,7 @@
         <v>68</v>
       </c>
       <c r="AG23" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="AM23">
         <f t="shared" si="12"/>
@@ -6112,7 +6116,7 @@
         <v>C1MT-C2MT-O1MT</v>
       </c>
       <c r="AU23" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="AV23">
         <v>21</v>
@@ -6129,10 +6133,10 @@
         <v>68</v>
       </c>
       <c r="AZ23" s="7" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="BA23" s="7" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="BE23">
         <f t="shared" si="13"/>
@@ -6171,7 +6175,7 @@
         <v>NMT-SMT-C1MT-HMT</v>
       </c>
       <c r="BP23" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ23">
         <v>21</v>
@@ -6196,7 +6200,7 @@
         <v>68</v>
       </c>
       <c r="BW23" s="8" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="BX23" s="8" t="str">
         <f>"Same as "&amp;BW12</f>
@@ -6232,10 +6236,10 @@
         <v>68</v>
       </c>
       <c r="I24" s="15" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="K24" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="L24">
         <f t="shared" si="2"/>
@@ -6290,7 +6294,7 @@
         <v>C1MT-C1MT-C1MT</v>
       </c>
       <c r="AU24" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="AV24">
         <v>22</v>
@@ -6307,10 +6311,10 @@
         <v>68</v>
       </c>
       <c r="AZ24" s="7" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="BA24" s="7" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="BE24">
         <f t="shared" si="13"/>
@@ -6349,7 +6353,7 @@
         <v>O2MT-C2MT-C1MT-C1MT</v>
       </c>
       <c r="BP24" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ24">
         <v>22</v>
@@ -6374,7 +6378,7 @@
         <v>68</v>
       </c>
       <c r="BW24" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="BX24" t="str">
         <f t="shared" ref="BX24" si="24">BW24</f>
@@ -6384,7 +6388,7 @@
     <row r="25" spans="2:76" x14ac:dyDescent="0.25">
       <c r="M25" s="9"/>
       <c r="AC25" s="16" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AM25">
         <f t="shared" si="12"/>
@@ -6415,7 +6419,7 @@
         <v>SMT-NMT-SMT</v>
       </c>
       <c r="AU25" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="AV25">
         <v>23</v>
@@ -6432,7 +6436,7 @@
         <v>68</v>
       </c>
       <c r="AZ25" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="BE25">
         <f t="shared" si="13"/>
@@ -6471,7 +6475,7 @@
         <v>O2MT-C2MT-C1MT-HMT</v>
       </c>
       <c r="BP25" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ25">
         <v>23</v>
@@ -6496,10 +6500,10 @@
         <v>68</v>
       </c>
       <c r="BW25" s="7" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="BX25" s="7" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
     </row>
     <row r="26" spans="2:76" x14ac:dyDescent="0.25">
@@ -6533,7 +6537,7 @@
         <v>C2MT-O1MT-C1MT</v>
       </c>
       <c r="AU26" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="AV26">
         <v>24</v>
@@ -6550,7 +6554,7 @@
         <v>68</v>
       </c>
       <c r="AZ26" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="BE26">
         <f t="shared" si="13"/>
@@ -6589,7 +6593,7 @@
         <v>O1MT-C2MT-C1MT-C1MT</v>
       </c>
       <c r="BP26" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ26">
         <v>24</v>
@@ -6614,10 +6618,10 @@
         <v>68</v>
       </c>
       <c r="BW26" s="7" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="BX26" s="7" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
     </row>
     <row r="27" spans="2:76" x14ac:dyDescent="0.25">
@@ -6651,7 +6655,7 @@
         <v>O3MT-SMT-O3MT</v>
       </c>
       <c r="AU27" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="AV27">
         <v>25</v>
@@ -6668,7 +6672,7 @@
         <v>68</v>
       </c>
       <c r="AZ27" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="BE27">
         <f t="shared" si="13"/>
@@ -6707,7 +6711,7 @@
         <v>O1MT-C2MT-C1MT-HMT</v>
       </c>
       <c r="BP27" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ27">
         <v>25</v>
@@ -6732,7 +6736,7 @@
         <v>68</v>
       </c>
       <c r="BW27" s="7" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="BX27" s="7" t="str">
         <f>"Same as "&amp;BW11</f>
@@ -6741,7 +6745,7 @@
     </row>
     <row r="28" spans="2:76" x14ac:dyDescent="0.25">
       <c r="F28" s="20" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="G28" s="20"/>
       <c r="H28" s="20"/>
@@ -6776,7 +6780,7 @@
         <v>C1MT-C2MT-O2MT</v>
       </c>
       <c r="AU28" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="AV28">
         <v>26</v>
@@ -6793,7 +6797,7 @@
         <v>68</v>
       </c>
       <c r="AZ28" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="BE28">
         <f t="shared" si="13"/>
@@ -6832,7 +6836,7 @@
         <v>O3MT-SMT-C1MT-C1MT</v>
       </c>
       <c r="BP28" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ28">
         <v>26</v>
@@ -6857,7 +6861,7 @@
         <v>68</v>
       </c>
       <c r="BW28" s="7" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="BX28" s="7" t="str">
         <f>"Same as "&amp;BW16</f>
@@ -6895,7 +6899,7 @@
         <v>O1MT-C2MT-O2MT</v>
       </c>
       <c r="AU29" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="AV29">
         <v>27</v>
@@ -6912,7 +6916,7 @@
         <v>68</v>
       </c>
       <c r="AZ29" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="BE29">
         <f t="shared" si="13"/>
@@ -6951,7 +6955,7 @@
         <v>O3MT-SMT-C1MT-HMT</v>
       </c>
       <c r="BP29" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ29">
         <v>27</v>
@@ -6976,7 +6980,7 @@
         <v>68</v>
       </c>
       <c r="BW29" s="7" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="BX29" s="7" t="str">
         <f>"Same as "&amp;BW17</f>
@@ -7012,7 +7016,7 @@
         <v>#</v>
       </c>
       <c r="I30" s="17" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="M30" s="9"/>
       <c r="AM30">
@@ -7044,7 +7048,7 @@
         <v>HV-C1V-HV</v>
       </c>
       <c r="AU30" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="AV30">
         <v>28</v>
@@ -7061,7 +7065,7 @@
         <v>68</v>
       </c>
       <c r="AZ30" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="BE30">
         <f t="shared" si="13"/>
@@ -7100,7 +7104,7 @@
         <v>O3MT-SMT-NMT-SMT</v>
       </c>
       <c r="BP30" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ30">
         <v>28</v>
@@ -7125,12 +7129,12 @@
         <v>68</v>
       </c>
       <c r="BW30" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
     </row>
     <row r="31" spans="2:76" x14ac:dyDescent="0.25">
       <c r="B31" s="17" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="C31" s="17">
         <f>E30</f>
@@ -7187,7 +7191,7 @@
         <v>O1V-C1V-HV</v>
       </c>
       <c r="AU31" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="AV31" s="16">
         <v>29</v>
@@ -7204,7 +7208,7 @@
         <v>68</v>
       </c>
       <c r="AZ31" s="16" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="BE31">
         <f t="shared" si="13"/>
@@ -7243,7 +7247,7 @@
         <v>SMT-C1MT-C1MT-C1MT</v>
       </c>
       <c r="BP31" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ31">
         <v>29</v>
@@ -7268,7 +7272,7 @@
         <v>68</v>
       </c>
       <c r="BW31" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
     </row>
     <row r="32" spans="2:76" x14ac:dyDescent="0.25">
@@ -7302,7 +7306,7 @@
         <v>HV-C1V-C1V</v>
       </c>
       <c r="AU32" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="AV32">
         <v>30</v>
@@ -7319,7 +7323,7 @@
         <v>68</v>
       </c>
       <c r="AZ32" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="BE32">
         <f t="shared" si="13"/>
@@ -7358,7 +7362,7 @@
         <v>SMT-C1MT-C1MT-HMT</v>
       </c>
       <c r="BP32" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ32">
         <v>30</v>
@@ -7383,7 +7387,7 @@
         <v>68</v>
       </c>
       <c r="BW32" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
     </row>
     <row r="33" spans="13:76" x14ac:dyDescent="0.25">
@@ -7417,7 +7421,7 @@
         <v>C1V-C1V-O1V</v>
       </c>
       <c r="AU33" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="AV33">
         <v>31</v>
@@ -7434,7 +7438,7 @@
         <v>68</v>
       </c>
       <c r="AZ33" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="BE33">
         <f t="shared" si="13"/>
@@ -7473,7 +7477,7 @@
         <v>SMT-NMT-SMT-C1MT</v>
       </c>
       <c r="BP33" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ33">
         <v>31</v>
@@ -7498,7 +7502,7 @@
         <v>68</v>
       </c>
       <c r="BW33" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
     </row>
     <row r="34" spans="13:76" x14ac:dyDescent="0.25">
@@ -7532,7 +7536,7 @@
         <v>C1V-C1V-C1V</v>
       </c>
       <c r="AU34" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="AV34">
         <v>32</v>
@@ -7549,7 +7553,7 @@
         <v>68</v>
       </c>
       <c r="AZ34" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="BE34">
         <f t="shared" si="13"/>
@@ -7588,7 +7592,7 @@
         <v>C2V-O1V-C1V-C1V</v>
       </c>
       <c r="BP34" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ34">
         <v>32</v>
@@ -7613,7 +7617,7 @@
         <v>68</v>
       </c>
       <c r="BW34" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
     </row>
     <row r="35" spans="13:76" x14ac:dyDescent="0.25">
@@ -7647,7 +7651,7 @@
         <v>O1V-C2V-O1V</v>
       </c>
       <c r="AU35" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="AV35" s="16">
         <v>33</v>
@@ -7664,7 +7668,7 @@
         <v>68</v>
       </c>
       <c r="AZ35" s="16" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="BE35">
         <f t="shared" si="13"/>
@@ -7703,7 +7707,7 @@
         <v>O1V-C1V-C1V-O1V</v>
       </c>
       <c r="BP35" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ35">
         <v>33</v>
@@ -7728,10 +7732,10 @@
         <v>68</v>
       </c>
       <c r="BW35" s="7" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="BX35" s="7" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
     </row>
     <row r="36" spans="13:76" x14ac:dyDescent="0.25">
@@ -7765,7 +7769,7 @@
         <v>C1V-O1V-C2V</v>
       </c>
       <c r="AU36" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="AV36">
         <v>34</v>
@@ -7782,7 +7786,7 @@
         <v>68</v>
       </c>
       <c r="AZ36" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="BE36">
         <f t="shared" si="13"/>
@@ -7821,7 +7825,7 @@
         <v>C2V-O1V-C1V-HV</v>
       </c>
       <c r="BP36" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ36">
         <v>34</v>
@@ -7846,7 +7850,7 @@
         <v>68</v>
       </c>
       <c r="BW36" s="7" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="BX36" s="7" t="str">
         <f>"Same as "&amp;BW34</f>
@@ -7884,7 +7888,7 @@
         <v>O1V-C2V-O2V</v>
       </c>
       <c r="AU37" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="AV37">
         <v>35</v>
@@ -7901,7 +7905,7 @@
         <v>68</v>
       </c>
       <c r="AZ37" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="BE37">
         <f t="shared" si="13"/>
@@ -7940,7 +7944,7 @@
         <v>C1V-C1V-C1V-HV</v>
       </c>
       <c r="BP37" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ37">
         <v>35</v>
@@ -7965,13 +7969,13 @@
         <v>68</v>
       </c>
       <c r="BW37" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
     </row>
     <row r="38" spans="13:76" x14ac:dyDescent="0.25">
       <c r="M38" s="9"/>
       <c r="AU38" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="AV38">
         <v>36</v>
@@ -7988,7 +7992,7 @@
         <v>68</v>
       </c>
       <c r="AZ38" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="BE38">
         <f t="shared" si="13"/>
@@ -8027,7 +8031,7 @@
         <v>HV-C1V-C1V-HV</v>
       </c>
       <c r="BP38" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ38">
         <v>36</v>
@@ -8052,13 +8056,13 @@
         <v>68</v>
       </c>
       <c r="BW38" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
     </row>
     <row r="39" spans="13:76" x14ac:dyDescent="0.25">
       <c r="M39" s="9"/>
       <c r="AU39" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="AV39">
         <v>37</v>
@@ -8075,7 +8079,7 @@
         <v>68</v>
       </c>
       <c r="AZ39" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="BE39">
         <f t="shared" si="13"/>
@@ -8114,7 +8118,7 @@
         <v>HV-C1V-C1V-O1V</v>
       </c>
       <c r="BP39" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ39">
         <v>37</v>
@@ -8139,13 +8143,13 @@
         <v>68</v>
       </c>
       <c r="BW39" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
     </row>
     <row r="40" spans="13:76" x14ac:dyDescent="0.25">
       <c r="M40" s="9"/>
       <c r="AU40" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="AV40">
         <v>38</v>
@@ -8162,7 +8166,7 @@
         <v>68</v>
       </c>
       <c r="AZ40" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="BE40">
         <f t="shared" si="13"/>
@@ -8201,7 +8205,7 @@
         <v>C1V-C1V-C1V-C1V</v>
       </c>
       <c r="BP40" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ40">
         <v>38</v>
@@ -8226,13 +8230,13 @@
         <v>68</v>
       </c>
       <c r="BW40" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
     </row>
     <row r="41" spans="13:76" x14ac:dyDescent="0.25">
       <c r="M41" s="9"/>
       <c r="AU41" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="AV41">
         <v>39</v>
@@ -8249,7 +8253,7 @@
         <v>68</v>
       </c>
       <c r="AZ41" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="BE41">
         <f t="shared" si="13"/>
@@ -8288,7 +8292,7 @@
         <v>O1V-C1V-C1V-C1V</v>
       </c>
       <c r="BP41" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ41">
         <v>39</v>
@@ -8313,7 +8317,7 @@
         <v>68</v>
       </c>
       <c r="BW41" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
     </row>
     <row r="42" spans="13:76" x14ac:dyDescent="0.25">
@@ -8355,7 +8359,7 @@
         <v>O2V-C2V-O1V-C1V</v>
       </c>
       <c r="BP42" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ42">
         <v>40</v>
@@ -8380,7 +8384,7 @@
         <v>68</v>
       </c>
       <c r="BW42" s="7" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="BX42" s="7" t="str">
         <f>"Same as "&amp;BW31</f>
@@ -8426,7 +8430,7 @@
         <v>C1V-O1V-C2V-O1V</v>
       </c>
       <c r="BP43" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ43">
         <v>41</v>
@@ -8451,7 +8455,7 @@
         <v>68</v>
       </c>
       <c r="BW43" s="7" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="BX43" s="7" t="str">
         <f>"Same as "&amp;BW39</f>
@@ -8461,7 +8465,7 @@
     <row r="44" spans="13:76" x14ac:dyDescent="0.25">
       <c r="M44" s="9"/>
       <c r="BP44" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ44">
         <v>42</v>
@@ -8486,13 +8490,13 @@
         <v>68</v>
       </c>
       <c r="BW44" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
     </row>
     <row r="45" spans="13:76" x14ac:dyDescent="0.25">
       <c r="M45" s="9"/>
       <c r="BP45" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ45">
         <v>43</v>
@@ -8517,13 +8521,13 @@
         <v>68</v>
       </c>
       <c r="BW45" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
     </row>
     <row r="46" spans="13:76" x14ac:dyDescent="0.25">
       <c r="M46" s="9"/>
       <c r="BP46" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ46">
         <v>44</v>
@@ -8548,13 +8552,13 @@
         <v>68</v>
       </c>
       <c r="BW46" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
     </row>
     <row r="47" spans="13:76" x14ac:dyDescent="0.25">
       <c r="M47" s="9"/>
       <c r="BP47" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ47">
         <v>45</v>
@@ -8579,13 +8583,13 @@
         <v>68</v>
       </c>
       <c r="BW47" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
     </row>
     <row r="48" spans="13:76" x14ac:dyDescent="0.25">
       <c r="M48" s="9"/>
       <c r="BP48" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ48">
         <v>46</v>
@@ -8610,12 +8614,12 @@
         <v>68</v>
       </c>
       <c r="BW48" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
     </row>
     <row r="49" spans="68:75" x14ac:dyDescent="0.25">
       <c r="BP49" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ49">
         <v>47</v>
@@ -8640,12 +8644,12 @@
         <v>68</v>
       </c>
       <c r="BW49" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
     </row>
     <row r="50" spans="68:75" x14ac:dyDescent="0.25">
       <c r="BP50" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ50">
         <v>48</v>
@@ -8670,12 +8674,12 @@
         <v>68</v>
       </c>
       <c r="BW50" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
     </row>
     <row r="51" spans="68:75" x14ac:dyDescent="0.25">
       <c r="BP51" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ51">
         <v>49</v>
@@ -8700,12 +8704,12 @@
         <v>68</v>
       </c>
       <c r="BW51" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
     </row>
     <row r="52" spans="68:75" x14ac:dyDescent="0.25">
       <c r="BP52" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ52">
         <v>50</v>
@@ -8730,12 +8734,12 @@
         <v>68</v>
       </c>
       <c r="BW52" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
     </row>
     <row r="53" spans="68:75" x14ac:dyDescent="0.25">
       <c r="BP53" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ53">
         <v>51</v>
@@ -8760,12 +8764,12 @@
         <v>68</v>
       </c>
       <c r="BW53" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
     </row>
     <row r="54" spans="68:75" x14ac:dyDescent="0.25">
       <c r="BP54" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ54">
         <v>52</v>
@@ -8790,12 +8794,12 @@
         <v>68</v>
       </c>
       <c r="BW54" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
     </row>
     <row r="55" spans="68:75" x14ac:dyDescent="0.25">
       <c r="BP55" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="BQ55">
         <v>53</v>
@@ -8820,17 +8824,17 @@
         <v>68</v>
       </c>
       <c r="BW55" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
     </row>
     <row r="61" spans="68:75" x14ac:dyDescent="0.25">
       <c r="BQ61" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
     </row>
     <row r="62" spans="68:75" x14ac:dyDescent="0.25">
       <c r="BQ62" s="7" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="BR62" s="7">
         <v>1.3</v>
@@ -8848,12 +8852,12 @@
         <v>68</v>
       </c>
       <c r="BW62" s="7" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
     </row>
     <row r="63" spans="68:75" x14ac:dyDescent="0.25">
       <c r="BQ63" s="7" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="BR63" s="7">
         <v>-2.06</v>
@@ -8871,7 +8875,7 @@
         <v>68</v>
       </c>
       <c r="BW63" s="7" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
     </row>
   </sheetData>
@@ -32797,7 +32801,7 @@
     </row>
     <row r="53" spans="1:39" ht="75" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B53" s="1" t="s">
         <v>27</v>
@@ -32864,7 +32868,7 @@
         <v>18</v>
       </c>
       <c r="N54" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="P54" t="s">
         <v>68</v>

</xml_diff>